<commit_message>
chore: persist RAVIQO bot state
</commit_message>
<xml_diff>
--- a/data/logs.xlsx
+++ b/data/logs.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N178"/>
+  <dimension ref="A1:N264"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -10081,7 +10081,6 @@
           <t>https://x.com/adrianflynn/status/2100171382734684530</t>
         </is>
       </c>
-      <c r="G178" t="inlineStr"/>
       <c r="H178" t="n">
         <v>0</v>
       </c>
@@ -10093,16 +10092,4686 @@
           <t>multi_group</t>
         </is>
       </c>
-      <c r="K178" t="inlineStr"/>
       <c r="L178" t="inlineStr">
         <is>
           <t>ERROR</t>
         </is>
       </c>
-      <c r="M178" t="inlineStr"/>
       <c r="N178" t="inlineStr">
         <is>
           <t>Error code: 401 - {'error': {'message': 'Incorrect API key provided: AQ.Ab8RN*****************************************PQsA. You can find your API key at https://platform.openai.com/account/api-keys.', 'type': 'invalid_request_error', 'param': None, 'code': 'invalid_api_key'}}</t>
+        </is>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B179" t="inlineStr">
+        <is>
+          <t>10:52:59</t>
+        </is>
+      </c>
+      <c r="C179" t="inlineStr">
+        <is>
+          <t>2100175875878633970</t>
+        </is>
+      </c>
+      <c r="D179" t="inlineStr">
+        <is>
+          <t>redbat75</t>
+        </is>
+      </c>
+      <c r="E179" t="inlineStr">
+        <is>
+          <t>If every experience ends in the founder’s head, the founder is learning.
+The business isn’t.</t>
+        </is>
+      </c>
+      <c r="F179" t="inlineStr">
+        <is>
+          <t>https://x.com/redbat75/status/2100175875878633970</t>
+        </is>
+      </c>
+      <c r="H179" t="n">
+        <v>0</v>
+      </c>
+      <c r="I179" t="n">
+        <v>0</v>
+      </c>
+      <c r="J179" t="inlineStr">
+        <is>
+          <t>multi_group</t>
+        </is>
+      </c>
+      <c r="L179" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="N179" t="inlineStr">
+        <is>
+          <t>Error code: 401 - [{'error': {'code': 401, 'message': 'Request had invalid authentication credentials. Expected OAuth 2 access token, login cookie or other valid authentication credential. See https://developers.google.com/identity/sign-in/web/devconsole-project.', 'status': 'UNAUTHENTICATED', 'details': [{'@type': 'type.googleapis.com/google.rpc.ErrorInfo', 'reason': 'ACCESS_TOKEN_TYPE_UNSUPPORTED', 'metadata': {'method': 'google.ai.generativelanguage.v1main.GenerativeService.GenerateContent', 'service': 'generativelanguage.googleapis.com'}}]}}]</t>
+        </is>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B180" t="inlineStr">
+        <is>
+          <t>10:52:59</t>
+        </is>
+      </c>
+      <c r="C180" t="inlineStr">
+        <is>
+          <t>2100175971961704564</t>
+        </is>
+      </c>
+      <c r="D180" t="inlineStr">
+        <is>
+          <t>Lang_Enthused</t>
+        </is>
+      </c>
+      <c r="E180" t="inlineStr">
+        <is>
+          <t>@DaffyGiving @adamnash @DaffyGiving @adamnash Classic founder answer 😄 fair. My hunch is the donation rate chart alone moves the needle, nobody wants to stare at a 0%. Would love to see aggregate before/after numbers in a year</t>
+        </is>
+      </c>
+      <c r="F180" t="inlineStr">
+        <is>
+          <t>https://x.com/Lang_Enthused/status/2100175971961704564</t>
+        </is>
+      </c>
+      <c r="H180" t="n">
+        <v>0</v>
+      </c>
+      <c r="I180" t="n">
+        <v>0</v>
+      </c>
+      <c r="J180" t="inlineStr">
+        <is>
+          <t>multi_group</t>
+        </is>
+      </c>
+      <c r="L180" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="N180" t="inlineStr">
+        <is>
+          <t>Error code: 401 - [{'error': {'code': 401, 'message': 'Request had invalid authentication credentials. Expected OAuth 2 access token, login cookie or other valid authentication credential. See https://developers.google.com/identity/sign-in/web/devconsole-project.', 'status': 'UNAUTHENTICATED', 'details': [{'@type': 'type.googleapis.com/google.rpc.ErrorInfo', 'reason': 'ACCESS_TOKEN_TYPE_UNSUPPORTED', 'metadata': {'method': 'google.ai.generativelanguage.v1main.GenerativeService.GenerateContent', 'service': 'generativelanguage.googleapis.com'}}]}}]</t>
+        </is>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B181" t="inlineStr">
+        <is>
+          <t>10:53:00</t>
+        </is>
+      </c>
+      <c r="C181" t="inlineStr">
+        <is>
+          <t>2100175966081290326</t>
+        </is>
+      </c>
+      <c r="D181" t="inlineStr">
+        <is>
+          <t>SulkaMike</t>
+        </is>
+      </c>
+      <c r="E181" t="inlineStr">
+        <is>
+          <t>Interesting hand we've been dealt this Wednesday morning. Google shipped a voice agent that can keep talking while it thinks, and a startup founded by one of the people behind the original ChatGPT research shipped an AI model that basically refuses to talk at all.
+Gemini 3.8</t>
+        </is>
+      </c>
+      <c r="F181" t="inlineStr">
+        <is>
+          <t>https://x.com/SulkaMike/status/2100175966081290326</t>
+        </is>
+      </c>
+      <c r="H181" t="n">
+        <v>0</v>
+      </c>
+      <c r="I181" t="n">
+        <v>0</v>
+      </c>
+      <c r="J181" t="inlineStr">
+        <is>
+          <t>multi_group</t>
+        </is>
+      </c>
+      <c r="L181" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="N181" t="inlineStr">
+        <is>
+          <t>Error code: 401 - [{'error': {'code': 401, 'message': 'Request had invalid authentication credentials. Expected OAuth 2 access token, login cookie or other valid authentication credential. See https://developers.google.com/identity/sign-in/web/devconsole-project.', 'status': 'UNAUTHENTICATED', 'details': [{'@type': 'type.googleapis.com/google.rpc.ErrorInfo', 'reason': 'ACCESS_TOKEN_TYPE_UNSUPPORTED', 'metadata': {'method': 'google.ai.generativelanguage.v1main.GenerativeService.GenerateContent', 'service': 'generativelanguage.googleapis.com'}}]}}]</t>
+        </is>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B182" t="inlineStr">
+        <is>
+          <t>10:53:00</t>
+        </is>
+      </c>
+      <c r="C182" t="inlineStr">
+        <is>
+          <t>2100175961962504383</t>
+        </is>
+      </c>
+      <c r="D182" t="inlineStr">
+        <is>
+          <t>Dannydev784</t>
+        </is>
+      </c>
+      <c r="E182" t="inlineStr">
+        <is>
+          <t>@berkaybakac Would be happy to connect. I am the solo founder of https://t.co/2JHQiJ6L1X Let’s grow together!</t>
+        </is>
+      </c>
+      <c r="F182" t="inlineStr">
+        <is>
+          <t>https://x.com/Dannydev784/status/2100175961962504383</t>
+        </is>
+      </c>
+      <c r="H182" t="n">
+        <v>0</v>
+      </c>
+      <c r="I182" t="n">
+        <v>0</v>
+      </c>
+      <c r="J182" t="inlineStr">
+        <is>
+          <t>multi_group</t>
+        </is>
+      </c>
+      <c r="L182" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="N182" t="inlineStr">
+        <is>
+          <t>Error code: 401 - [{'error': {'code': 401, 'message': 'Request had invalid authentication credentials. Expected OAuth 2 access token, login cookie or other valid authentication credential. See https://developers.google.com/identity/sign-in/web/devconsole-project.', 'status': 'UNAUTHENTICATED', 'details': [{'@type': 'type.googleapis.com/google.rpc.ErrorInfo', 'reason': 'ACCESS_TOKEN_TYPE_UNSUPPORTED', 'metadata': {'method': 'google.ai.generativelanguage.v1main.GenerativeService.GenerateContent', 'service': 'generativelanguage.googleapis.com'}}]}}]</t>
+        </is>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B183" t="inlineStr">
+        <is>
+          <t>10:53:00</t>
+        </is>
+      </c>
+      <c r="C183" t="inlineStr">
+        <is>
+          <t>2100175922305327546</t>
+        </is>
+      </c>
+      <c r="D183" t="inlineStr">
+        <is>
+          <t>TechMoran</t>
+        </is>
+      </c>
+      <c r="E183" t="inlineStr">
+        <is>
+          <t>Egyptian payments startup Zeal has raised $10M to take its technology global.The fresh capital will help the company roll out across more than 4 million payment terminals covered by signed contracts.
+That takes Zeal’s total funding to $14M.
+https://t.co/ykcumcToMq https://t.co/foQHfhPN5R</t>
+        </is>
+      </c>
+      <c r="F183" t="inlineStr">
+        <is>
+          <t>https://x.com/TechMoran/status/2100175922305327546</t>
+        </is>
+      </c>
+      <c r="H183" t="n">
+        <v>0</v>
+      </c>
+      <c r="I183" t="n">
+        <v>0</v>
+      </c>
+      <c r="J183" t="inlineStr">
+        <is>
+          <t>multi_group</t>
+        </is>
+      </c>
+      <c r="L183" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="N183" t="inlineStr">
+        <is>
+          <t>Error code: 401 - [{'error': {'code': 401, 'message': 'Request had invalid authentication credentials. Expected OAuth 2 access token, login cookie or other valid authentication credential. See https://developers.google.com/identity/sign-in/web/devconsole-project.', 'status': 'UNAUTHENTICATED', 'details': [{'@type': 'type.googleapis.com/google.rpc.ErrorInfo', 'reason': 'ACCESS_TOKEN_TYPE_UNSUPPORTED', 'metadata': {'method': 'google.ai.generativelanguage.v1main.GenerativeService.GenerateContent', 'service': 'generativelanguage.googleapis.com'}}]}}]</t>
+        </is>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B184" t="inlineStr">
+        <is>
+          <t>10:53:00</t>
+        </is>
+      </c>
+      <c r="C184" t="inlineStr">
+        <is>
+          <t>2100175906438299845</t>
+        </is>
+      </c>
+      <c r="D184" t="inlineStr">
+        <is>
+          <t>semiii</t>
+        </is>
+      </c>
+      <c r="E184" t="inlineStr">
+        <is>
+          <t>Startup Village Borneo was a super success. We got lots of budding talent from US, europe, singapore, vietnam, nepal, korea, india, indonesia, canada, ukraine, russia, and of course, West Malaysia.
+Check out all of their projects in the Borneo Builders Directory. https://t.co/2UBnG0ivjH</t>
+        </is>
+      </c>
+      <c r="F184" t="inlineStr">
+        <is>
+          <t>https://x.com/semiii/status/2100175906438299845</t>
+        </is>
+      </c>
+      <c r="H184" t="n">
+        <v>0</v>
+      </c>
+      <c r="I184" t="n">
+        <v>0</v>
+      </c>
+      <c r="J184" t="inlineStr">
+        <is>
+          <t>multi_group</t>
+        </is>
+      </c>
+      <c r="L184" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="N184" t="inlineStr">
+        <is>
+          <t>Error code: 401 - [{'error': {'code': 401, 'message': 'Request had invalid authentication credentials. Expected OAuth 2 access token, login cookie or other valid authentication credential. See https://developers.google.com/identity/sign-in/web/devconsole-project.', 'status': 'UNAUTHENTICATED', 'details': [{'@type': 'type.googleapis.com/google.rpc.ErrorInfo', 'reason': 'ACCESS_TOKEN_TYPE_UNSUPPORTED', 'metadata': {'method': 'google.ai.generativelanguage.v1main.GenerativeService.GenerateContent', 'service': 'generativelanguage.googleapis.com'}}]}}]</t>
+        </is>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B185" t="inlineStr">
+        <is>
+          <t>10:53:00</t>
+        </is>
+      </c>
+      <c r="C185" t="inlineStr">
+        <is>
+          <t>2100175896145531266</t>
+        </is>
+      </c>
+      <c r="D185" t="inlineStr">
+        <is>
+          <t>Mudhaxk</t>
+        </is>
+      </c>
+      <c r="E185" t="inlineStr">
+        <is>
+          <t>@rant_zine Hey, solo founder building here too. One of our early users (GreatmindsNG) cut about $90/month after moving backend, storage and email onto one platform - worth a look if you're juggling separate vendors for that stuff. https://t.co/L4AC6nUiDS</t>
+        </is>
+      </c>
+      <c r="F185" t="inlineStr">
+        <is>
+          <t>https://x.com/Mudhaxk/status/2100175896145531266</t>
+        </is>
+      </c>
+      <c r="H185" t="n">
+        <v>1</v>
+      </c>
+      <c r="I185" t="n">
+        <v>0</v>
+      </c>
+      <c r="J185" t="inlineStr">
+        <is>
+          <t>multi_group</t>
+        </is>
+      </c>
+      <c r="L185" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="N185" t="inlineStr">
+        <is>
+          <t>Error code: 401 - [{'error': {'code': 401, 'message': 'Request had invalid authentication credentials. Expected OAuth 2 access token, login cookie or other valid authentication credential. See https://developers.google.com/identity/sign-in/web/devconsole-project.', 'status': 'UNAUTHENTICATED', 'details': [{'@type': 'type.googleapis.com/google.rpc.ErrorInfo', 'reason': 'ACCESS_TOKEN_TYPE_UNSUPPORTED', 'metadata': {'method': 'google.ai.generativelanguage.v1main.GenerativeService.GenerateContent', 'service': 'generativelanguage.googleapis.com'}}]}}]</t>
+        </is>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B186" t="inlineStr">
+        <is>
+          <t>10:53:00</t>
+        </is>
+      </c>
+      <c r="C186" t="inlineStr">
+        <is>
+          <t>2100175903217070532</t>
+        </is>
+      </c>
+      <c r="D186" t="inlineStr">
+        <is>
+          <t>kelvonhimself</t>
+        </is>
+      </c>
+      <c r="E186" t="inlineStr">
+        <is>
+          <t>$0 → $100k/day - Day 83
+First day after being back in stock, feeling that back in stock hangover way early this time. Ads spent at a terrible efficiency which sucks.
+My quiz funnel is working okay for now, further optimization is needed. Currently sitting at 20% completion https://t.co/GznAOwOkSH</t>
+        </is>
+      </c>
+      <c r="F186" t="inlineStr">
+        <is>
+          <t>https://x.com/kelvonhimself/status/2100175903217070532</t>
+        </is>
+      </c>
+      <c r="H186" t="n">
+        <v>0</v>
+      </c>
+      <c r="I186" t="n">
+        <v>0</v>
+      </c>
+      <c r="J186" t="inlineStr">
+        <is>
+          <t>multi_group</t>
+        </is>
+      </c>
+      <c r="L186" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="N186" t="inlineStr">
+        <is>
+          <t>Error code: 401 - [{'error': {'code': 401, 'message': 'Request had invalid authentication credentials. Expected OAuth 2 access token, login cookie or other valid authentication credential. See https://developers.google.com/identity/sign-in/web/devconsole-project.', 'status': 'UNAUTHENTICATED', 'details': [{'@type': 'type.googleapis.com/google.rpc.ErrorInfo', 'reason': 'ACCESS_TOKEN_TYPE_UNSUPPORTED', 'metadata': {'service': 'generativelanguage.googleapis.com', 'method': 'google.ai.generativelanguage.v1main.GenerativeService.GenerateContent'}}]}}]</t>
+        </is>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B187" t="inlineStr">
+        <is>
+          <t>10:53:00</t>
+        </is>
+      </c>
+      <c r="C187" t="inlineStr">
+        <is>
+          <t>2100175890789384323</t>
+        </is>
+      </c>
+      <c r="D187" t="inlineStr">
+        <is>
+          <t>RichSementa</t>
+        </is>
+      </c>
+      <c r="E187" t="inlineStr">
+        <is>
+          <t>Palantir Co-Founder: Doomer Narratives on AI Are Ridiculous
+@JTLonsdale: So there’s lots of risks and there’s lots of upside but I think the doomer narratives are ridiculous and we should be embracing the industrial revolution."
+“Same thing they did with climate change and https://t.co/5MeAkFlWDj</t>
+        </is>
+      </c>
+      <c r="F187" t="inlineStr">
+        <is>
+          <t>https://x.com/RichSementa/status/2100175890789384323</t>
+        </is>
+      </c>
+      <c r="H187" t="n">
+        <v>0</v>
+      </c>
+      <c r="I187" t="n">
+        <v>0</v>
+      </c>
+      <c r="J187" t="inlineStr">
+        <is>
+          <t>multi_group</t>
+        </is>
+      </c>
+      <c r="L187" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="N187" t="inlineStr">
+        <is>
+          <t>Error code: 401 - [{'error': {'code': 401, 'message': 'Request had invalid authentication credentials. Expected OAuth 2 access token, login cookie or other valid authentication credential. See https://developers.google.com/identity/sign-in/web/devconsole-project.', 'status': 'UNAUTHENTICATED', 'details': [{'@type': 'type.googleapis.com/google.rpc.ErrorInfo', 'reason': 'ACCESS_TOKEN_TYPE_UNSUPPORTED', 'metadata': {'method': 'google.ai.generativelanguage.v1main.GenerativeService.GenerateContent', 'service': 'generativelanguage.googleapis.com'}}]}}]</t>
+        </is>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B188" t="inlineStr">
+        <is>
+          <t>10:53:00</t>
+        </is>
+      </c>
+      <c r="C188" t="inlineStr">
+        <is>
+          <t>2100175838788403496</t>
+        </is>
+      </c>
+      <c r="D188" t="inlineStr">
+        <is>
+          <t>REOComms</t>
+        </is>
+      </c>
+      <c r="E188" t="inlineStr">
+        <is>
+          <t>Ivorian group Kaydan plans to invest FCFA 500bn in fibre, housing and construction by 2030, while expanding into tech, cybersecurity and mining services. Founder @alainyaokouadio told us how this can create jobs and build Ivorian champions. #CotedIvoire 
+@FortuneMagazine https://t.co/mtmf5s8F3P</t>
+        </is>
+      </c>
+      <c r="F188" t="inlineStr">
+        <is>
+          <t>https://x.com/REOComms/status/2100175838788403496</t>
+        </is>
+      </c>
+      <c r="H188" t="n">
+        <v>0</v>
+      </c>
+      <c r="I188" t="n">
+        <v>0</v>
+      </c>
+      <c r="J188" t="inlineStr">
+        <is>
+          <t>multi_group</t>
+        </is>
+      </c>
+      <c r="L188" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="N188" t="inlineStr">
+        <is>
+          <t>Error code: 401 - [{'error': {'code': 401, 'message': 'Request had invalid authentication credentials. Expected OAuth 2 access token, login cookie or other valid authentication credential. See https://developers.google.com/identity/sign-in/web/devconsole-project.', 'status': 'UNAUTHENTICATED', 'details': [{'@type': 'type.googleapis.com/google.rpc.ErrorInfo', 'reason': 'ACCESS_TOKEN_TYPE_UNSUPPORTED', 'metadata': {'method': 'google.ai.generativelanguage.v1main.GenerativeService.GenerateContent', 'service': 'generativelanguage.googleapis.com'}}]}}]</t>
+        </is>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B189" t="inlineStr">
+        <is>
+          <t>10:53:00</t>
+        </is>
+      </c>
+      <c r="C189" t="inlineStr">
+        <is>
+          <t>2100175801769394657</t>
+        </is>
+      </c>
+      <c r="D189" t="inlineStr">
+        <is>
+          <t>NLAB_s</t>
+        </is>
+      </c>
+      <c r="E189" t="inlineStr">
+        <is>
+          <t>@giutheginger Solo Founder from Bcn too, Let’s connect</t>
+        </is>
+      </c>
+      <c r="F189" t="inlineStr">
+        <is>
+          <t>https://x.com/NLAB_s/status/2100175801769394657</t>
+        </is>
+      </c>
+      <c r="H189" t="n">
+        <v>0</v>
+      </c>
+      <c r="I189" t="n">
+        <v>0</v>
+      </c>
+      <c r="J189" t="inlineStr">
+        <is>
+          <t>multi_group</t>
+        </is>
+      </c>
+      <c r="L189" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="N189" t="inlineStr">
+        <is>
+          <t>Error code: 401 - [{'error': {'code': 401, 'message': 'Request had invalid authentication credentials. Expected OAuth 2 access token, login cookie or other valid authentication credential. See https://developers.google.com/identity/sign-in/web/devconsole-project.', 'status': 'UNAUTHENTICATED', 'details': [{'@type': 'type.googleapis.com/google.rpc.ErrorInfo', 'reason': 'ACCESS_TOKEN_TYPE_UNSUPPORTED', 'metadata': {'method': 'google.ai.generativelanguage.v1main.GenerativeService.GenerateContent', 'service': 'generativelanguage.googleapis.com'}}]}}]</t>
+        </is>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B190" t="inlineStr">
+        <is>
+          <t>10:53:00</t>
+        </is>
+      </c>
+      <c r="C190" t="inlineStr">
+        <is>
+          <t>2100175795524087850</t>
+        </is>
+      </c>
+      <c r="D190" t="inlineStr">
+        <is>
+          <t>Adom1063fm</t>
+        </is>
+      </c>
+      <c r="E190" t="inlineStr">
+        <is>
+          <t>NDC is doing well with regards to the macro-economy, but can they sustain it? - Alan Kyerematen (Founder and Leader, United Party)
+#DwasoNsem https://t.co/z7gOO6xNcP</t>
+        </is>
+      </c>
+      <c r="F190" t="inlineStr">
+        <is>
+          <t>https://x.com/Adom1063fm/status/2100175795524087850</t>
+        </is>
+      </c>
+      <c r="H190" t="n">
+        <v>0</v>
+      </c>
+      <c r="I190" t="n">
+        <v>0</v>
+      </c>
+      <c r="J190" t="inlineStr">
+        <is>
+          <t>multi_group</t>
+        </is>
+      </c>
+      <c r="L190" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="N190" t="inlineStr">
+        <is>
+          <t>Error code: 401 - [{'error': {'code': 401, 'message': 'Request had invalid authentication credentials. Expected OAuth 2 access token, login cookie or other valid authentication credential. See https://developers.google.com/identity/sign-in/web/devconsole-project.', 'status': 'UNAUTHENTICATED', 'details': [{'@type': 'type.googleapis.com/google.rpc.ErrorInfo', 'reason': 'ACCESS_TOKEN_TYPE_UNSUPPORTED', 'metadata': {'service': 'generativelanguage.googleapis.com', 'method': 'google.ai.generativelanguage.v1main.GenerativeService.GenerateContent'}}]}}]</t>
+        </is>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B191" t="inlineStr">
+        <is>
+          <t>10:53:01</t>
+        </is>
+      </c>
+      <c r="C191" t="inlineStr">
+        <is>
+          <t>2100175779975819664</t>
+        </is>
+      </c>
+      <c r="D191" t="inlineStr">
+        <is>
+          <t>Dannyzem3</t>
+        </is>
+      </c>
+      <c r="E191" t="inlineStr">
+        <is>
+          <t>@massivefanNWO @doveyymargeauxx I'm not talking about the donation to Reform.
+As the founder gets to set the charity's governing document, he can choose how trustees are selected, and select those who will pay him a wage. The £25m bank asset slowly becomes a wage expense, the books are balanced, but immorally.</t>
+        </is>
+      </c>
+      <c r="F191" t="inlineStr">
+        <is>
+          <t>https://x.com/Dannyzem3/status/2100175779975819664</t>
+        </is>
+      </c>
+      <c r="H191" t="n">
+        <v>0</v>
+      </c>
+      <c r="I191" t="n">
+        <v>0</v>
+      </c>
+      <c r="J191" t="inlineStr">
+        <is>
+          <t>multi_group</t>
+        </is>
+      </c>
+      <c r="L191" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="N191" t="inlineStr">
+        <is>
+          <t>Error code: 401 - [{'error': {'code': 401, 'message': 'Request had invalid authentication credentials. Expected OAuth 2 access token, login cookie or other valid authentication credential. See https://developers.google.com/identity/sign-in/web/devconsole-project.', 'status': 'UNAUTHENTICATED', 'details': [{'@type': 'type.googleapis.com/google.rpc.ErrorInfo', 'reason': 'ACCESS_TOKEN_TYPE_UNSUPPORTED', 'metadata': {'method': 'google.ai.generativelanguage.v1main.GenerativeService.GenerateContent', 'service': 'generativelanguage.googleapis.com'}}]}}]</t>
+        </is>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B192" t="inlineStr">
+        <is>
+          <t>10:53:01</t>
+        </is>
+      </c>
+      <c r="C192" t="inlineStr">
+        <is>
+          <t>2100175765430006255</t>
+        </is>
+      </c>
+      <c r="D192" t="inlineStr">
+        <is>
+          <t>prettyinpiece</t>
+        </is>
+      </c>
+      <c r="E192" t="inlineStr">
+        <is>
+          <t>I’m happy to officially announce to y’all that, with my ₦5,500, I am now in partnership with Dangote Group of Companies as a shareholder and co-founder. 
+Together, we’re working toward a better Nigeria! 🇳🇬 https://t.co/T4MbMw9vLt</t>
+        </is>
+      </c>
+      <c r="F192" t="inlineStr">
+        <is>
+          <t>https://x.com/prettyinpiece/status/2100175765430006255</t>
+        </is>
+      </c>
+      <c r="H192" t="n">
+        <v>0</v>
+      </c>
+      <c r="I192" t="n">
+        <v>0</v>
+      </c>
+      <c r="J192" t="inlineStr">
+        <is>
+          <t>multi_group</t>
+        </is>
+      </c>
+      <c r="L192" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="N192" t="inlineStr">
+        <is>
+          <t>Error code: 401 - [{'error': {'code': 401, 'message': 'Request had invalid authentication credentials. Expected OAuth 2 access token, login cookie or other valid authentication credential. See https://developers.google.com/identity/sign-in/web/devconsole-project.', 'status': 'UNAUTHENTICATED', 'details': [{'@type': 'type.googleapis.com/google.rpc.ErrorInfo', 'reason': 'ACCESS_TOKEN_TYPE_UNSUPPORTED', 'metadata': {'method': 'google.ai.generativelanguage.v1main.GenerativeService.GenerateContent', 'service': 'generativelanguage.googleapis.com'}}]}}]</t>
+        </is>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B193" t="inlineStr">
+        <is>
+          <t>10:53:01</t>
+        </is>
+      </c>
+      <c r="C193" t="inlineStr">
+        <is>
+          <t>2100175760061575250</t>
+        </is>
+      </c>
+      <c r="D193" t="inlineStr">
+        <is>
+          <t>geewon123</t>
+        </is>
+      </c>
+      <c r="E193" t="inlineStr">
+        <is>
+          <t>May Marvel film din kasi yata sila na kasabayan. Sana talaga maging successful kahit through word of mouth nalang yung marketing.</t>
+        </is>
+      </c>
+      <c r="F193" t="inlineStr">
+        <is>
+          <t>https://x.com/geewon123/status/2100175760061575250</t>
+        </is>
+      </c>
+      <c r="H193" t="n">
+        <v>0</v>
+      </c>
+      <c r="I193" t="n">
+        <v>0</v>
+      </c>
+      <c r="J193" t="inlineStr">
+        <is>
+          <t>multi_group</t>
+        </is>
+      </c>
+      <c r="L193" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="N193" t="inlineStr">
+        <is>
+          <t>Error code: 401 - [{'error': {'code': 401, 'message': 'Request had invalid authentication credentials. Expected OAuth 2 access token, login cookie or other valid authentication credential. See https://developers.google.com/identity/sign-in/web/devconsole-project.', 'status': 'UNAUTHENTICATED', 'details': [{'@type': 'type.googleapis.com/google.rpc.ErrorInfo', 'reason': 'ACCESS_TOKEN_TYPE_UNSUPPORTED', 'metadata': {'service': 'generativelanguage.googleapis.com', 'method': 'google.ai.generativelanguage.v1main.GenerativeService.GenerateContent'}}]}}]</t>
+        </is>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B194" t="inlineStr">
+        <is>
+          <t>10:53:01</t>
+        </is>
+      </c>
+      <c r="C194" t="inlineStr">
+        <is>
+          <t>2100175734622802027</t>
+        </is>
+      </c>
+      <c r="D194" t="inlineStr">
+        <is>
+          <t>carteiravazia</t>
+        </is>
+      </c>
+      <c r="E194" t="inlineStr">
+        <is>
+          <t>@burkov Eu tinha o mesmo pensamento que você, só que peguei costume de usar outras redes e deixei de usar o Facebook.
+Porém, não creio que a rede está morta, vejo muito conteúdo postado lá, tanto do feed páginas com dezenas de milhares de curtidas, pessoas, grupos, marketing place etc.</t>
+        </is>
+      </c>
+      <c r="F194" t="inlineStr">
+        <is>
+          <t>https://x.com/carteiravazia/status/2100175734622802027</t>
+        </is>
+      </c>
+      <c r="H194" t="n">
+        <v>0</v>
+      </c>
+      <c r="I194" t="n">
+        <v>0</v>
+      </c>
+      <c r="J194" t="inlineStr">
+        <is>
+          <t>multi_group</t>
+        </is>
+      </c>
+      <c r="L194" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="N194" t="inlineStr">
+        <is>
+          <t>Error code: 401 - [{'error': {'code': 401, 'message': 'Request had invalid authentication credentials. Expected OAuth 2 access token, login cookie or other valid authentication credential. See https://developers.google.com/identity/sign-in/web/devconsole-project.', 'status': 'UNAUTHENTICATED', 'details': [{'@type': 'type.googleapis.com/google.rpc.ErrorInfo', 'reason': 'ACCESS_TOKEN_TYPE_UNSUPPORTED', 'metadata': {'service': 'generativelanguage.googleapis.com', 'method': 'google.ai.generativelanguage.v1main.GenerativeService.GenerateContent'}}]}}]</t>
+        </is>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B195" t="inlineStr">
+        <is>
+          <t>10:53:01</t>
+        </is>
+      </c>
+      <c r="C195" t="inlineStr">
+        <is>
+          <t>2100175652544496020</t>
+        </is>
+      </c>
+      <c r="D195" t="inlineStr">
+        <is>
+          <t>T_E_Syndrome</t>
+        </is>
+      </c>
+      <c r="E195" t="inlineStr">
+        <is>
+          <t>@gummibear737 and they would be marketing that.... selling to everyone.</t>
+        </is>
+      </c>
+      <c r="F195" t="inlineStr">
+        <is>
+          <t>https://x.com/T_E_Syndrome/status/2100175652544496020</t>
+        </is>
+      </c>
+      <c r="H195" t="n">
+        <v>0</v>
+      </c>
+      <c r="I195" t="n">
+        <v>0</v>
+      </c>
+      <c r="J195" t="inlineStr">
+        <is>
+          <t>multi_group</t>
+        </is>
+      </c>
+      <c r="L195" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="N195" t="inlineStr">
+        <is>
+          <t>Error code: 401 - [{'error': {'code': 401, 'message': 'Request had invalid authentication credentials. Expected OAuth 2 access token, login cookie or other valid authentication credential. See https://developers.google.com/identity/sign-in/web/devconsole-project.', 'status': 'UNAUTHENTICATED', 'details': [{'@type': 'type.googleapis.com/google.rpc.ErrorInfo', 'reason': 'ACCESS_TOKEN_TYPE_UNSUPPORTED', 'metadata': {'method': 'google.ai.generativelanguage.v1main.GenerativeService.GenerateContent', 'service': 'generativelanguage.googleapis.com'}}]}}]</t>
+        </is>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B196" t="inlineStr">
+        <is>
+          <t>10:53:01</t>
+        </is>
+      </c>
+      <c r="C196" t="inlineStr">
+        <is>
+          <t>2100175616503120211</t>
+        </is>
+      </c>
+      <c r="D196" t="inlineStr">
+        <is>
+          <t>CdScissor</t>
+        </is>
+      </c>
+      <c r="E196" t="inlineStr">
+        <is>
+          <t>@Littleotomedius They're just really good at marketing, and sometimes it's warranted it's hard to argue against actual functional public transport.
+But I'd be lying if I said I'm not side-eyeing any questionable move the country makes. I know they've got history.
+Cute drawings tho</t>
+        </is>
+      </c>
+      <c r="F196" t="inlineStr">
+        <is>
+          <t>https://x.com/CdScissor/status/2100175616503120211</t>
+        </is>
+      </c>
+      <c r="H196" t="n">
+        <v>0</v>
+      </c>
+      <c r="I196" t="n">
+        <v>0</v>
+      </c>
+      <c r="J196" t="inlineStr">
+        <is>
+          <t>multi_group</t>
+        </is>
+      </c>
+      <c r="L196" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="N196" t="inlineStr">
+        <is>
+          <t>Error code: 401 - [{'error': {'code': 401, 'message': 'Request had invalid authentication credentials. Expected OAuth 2 access token, login cookie or other valid authentication credential. See https://developers.google.com/identity/sign-in/web/devconsole-project.', 'status': 'UNAUTHENTICATED', 'details': [{'@type': 'type.googleapis.com/google.rpc.ErrorInfo', 'reason': 'ACCESS_TOKEN_TYPE_UNSUPPORTED', 'metadata': {'method': 'google.ai.generativelanguage.v1main.GenerativeService.GenerateContent', 'service': 'generativelanguage.googleapis.com'}}]}}]</t>
+        </is>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B197" t="inlineStr">
+        <is>
+          <t>10:53:01</t>
+        </is>
+      </c>
+      <c r="C197" t="inlineStr">
+        <is>
+          <t>2100175612413390976</t>
+        </is>
+      </c>
+      <c r="D197" t="inlineStr">
+        <is>
+          <t>miroburn</t>
+        </is>
+      </c>
+      <c r="E197" t="inlineStr">
+        <is>
+          <t>Marketing z AI jest wyzwaniem.
+Ale jak się przepali odpowiednio dużo tokenów, doda dużo bramek i zrobi się kilka wtop, to nagle system zaczyna działać jak marzenie.
+Mój system składa się aktualnie z 18 podsystemów, które próbuję zrobić w 1 automat.
+Na razie najtrudniejsze https://t.co/Ryhsx1iHUu</t>
+        </is>
+      </c>
+      <c r="F197" t="inlineStr">
+        <is>
+          <t>https://x.com/miroburn/status/2100175612413390976</t>
+        </is>
+      </c>
+      <c r="H197" t="n">
+        <v>0</v>
+      </c>
+      <c r="I197" t="n">
+        <v>0</v>
+      </c>
+      <c r="J197" t="inlineStr">
+        <is>
+          <t>multi_group</t>
+        </is>
+      </c>
+      <c r="L197" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="N197" t="inlineStr">
+        <is>
+          <t>Error code: 401 - [{'error': {'code': 401, 'message': 'Request had invalid authentication credentials. Expected OAuth 2 access token, login cookie or other valid authentication credential. See https://developers.google.com/identity/sign-in/web/devconsole-project.', 'status': 'UNAUTHENTICATED', 'details': [{'@type': 'type.googleapis.com/google.rpc.ErrorInfo', 'reason': 'ACCESS_TOKEN_TYPE_UNSUPPORTED', 'metadata': {'method': 'google.ai.generativelanguage.v1main.GenerativeService.GenerateContent', 'service': 'generativelanguage.googleapis.com'}}]}}]</t>
+        </is>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B198" t="inlineStr">
+        <is>
+          <t>10:53:01</t>
+        </is>
+      </c>
+      <c r="C198" t="inlineStr">
+        <is>
+          <t>2100175600618975665</t>
+        </is>
+      </c>
+      <c r="D198" t="inlineStr">
+        <is>
+          <t>asaaseradio995</t>
+        </is>
+      </c>
+      <c r="E198" t="inlineStr">
+        <is>
+          <t>It is important to produce your own energy in your own country because it moves you from energy importation to energy sovereignty - Dr Riverson oppong- CEO of Chamber of oil Marketing Companies 
+#AsaaseBreakfastShow #Asaasenews #AsaaseRadio #AsaaseDigital https://t.co/3KDXZIlC9D</t>
+        </is>
+      </c>
+      <c r="F198" t="inlineStr">
+        <is>
+          <t>https://x.com/asaaseradio995/status/2100175600618975665</t>
+        </is>
+      </c>
+      <c r="H198" t="n">
+        <v>0</v>
+      </c>
+      <c r="I198" t="n">
+        <v>0</v>
+      </c>
+      <c r="J198" t="inlineStr">
+        <is>
+          <t>multi_group</t>
+        </is>
+      </c>
+      <c r="L198" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="N198" t="inlineStr">
+        <is>
+          <t>Error code: 401 - [{'error': {'code': 401, 'message': 'Request had invalid authentication credentials. Expected OAuth 2 access token, login cookie or other valid authentication credential. See https://developers.google.com/identity/sign-in/web/devconsole-project.', 'status': 'UNAUTHENTICATED', 'details': [{'@type': 'type.googleapis.com/google.rpc.ErrorInfo', 'reason': 'ACCESS_TOKEN_TYPE_UNSUPPORTED', 'metadata': {'method': 'google.ai.generativelanguage.v1main.GenerativeService.GenerateContent', 'service': 'generativelanguage.googleapis.com'}}]}}]</t>
+        </is>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B199" t="inlineStr">
+        <is>
+          <t>10:53:01</t>
+        </is>
+      </c>
+      <c r="C199" t="inlineStr">
+        <is>
+          <t>2100175577193885983</t>
+        </is>
+      </c>
+      <c r="D199" t="inlineStr">
+        <is>
+          <t>ricarcl</t>
+        </is>
+      </c>
+      <c r="E199" t="inlineStr">
+        <is>
+          <t>@Sfilmhead @KMbappe No es el mejor futbolista. Es el mejor goleador, que es diferente. El mejor futbolista es el que más facetas del juego abarca. 
+De hecho, con sus goles la temporada pasada, ni el Madrid ni la selección francesa ganaron nada. 
+El resto es marketing.</t>
+        </is>
+      </c>
+      <c r="F199" t="inlineStr">
+        <is>
+          <t>https://x.com/ricarcl/status/2100175577193885983</t>
+        </is>
+      </c>
+      <c r="H199" t="n">
+        <v>0</v>
+      </c>
+      <c r="I199" t="n">
+        <v>0</v>
+      </c>
+      <c r="J199" t="inlineStr">
+        <is>
+          <t>multi_group</t>
+        </is>
+      </c>
+      <c r="L199" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="N199" t="inlineStr">
+        <is>
+          <t>Error code: 401 - [{'error': {'code': 401, 'message': 'Request had invalid authentication credentials. Expected OAuth 2 access token, login cookie or other valid authentication credential. See https://developers.google.com/identity/sign-in/web/devconsole-project.', 'status': 'UNAUTHENTICATED', 'details': [{'@type': 'type.googleapis.com/google.rpc.ErrorInfo', 'reason': 'ACCESS_TOKEN_TYPE_UNSUPPORTED', 'metadata': {'method': 'google.ai.generativelanguage.v1main.GenerativeService.GenerateContent', 'service': 'generativelanguage.googleapis.com'}}]}}]</t>
+        </is>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B200" t="inlineStr">
+        <is>
+          <t>10:53:01</t>
+        </is>
+      </c>
+      <c r="C200" t="inlineStr">
+        <is>
+          <t>2100175576266936416</t>
+        </is>
+      </c>
+      <c r="D200" t="inlineStr">
+        <is>
+          <t>MeringueRouge</t>
+        </is>
+      </c>
+      <c r="E200" t="inlineStr">
+        <is>
+          <t>@SquireGrooktook Yeah I guess, but at least on social networks, there's that immediate recognition of what you're looking at that seems to be very important. In all my marketing, the best people recognised the game for was the big rack. That's it. It's a demon lady, but barely looks like a demon</t>
+        </is>
+      </c>
+      <c r="F200" t="inlineStr">
+        <is>
+          <t>https://x.com/MeringueRouge/status/2100175576266936416</t>
+        </is>
+      </c>
+      <c r="H200" t="n">
+        <v>0</v>
+      </c>
+      <c r="I200" t="n">
+        <v>0</v>
+      </c>
+      <c r="J200" t="inlineStr">
+        <is>
+          <t>multi_group</t>
+        </is>
+      </c>
+      <c r="L200" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="N200" t="inlineStr">
+        <is>
+          <t>Error code: 401 - [{'error': {'code': 401, 'message': 'Request had invalid authentication credentials. Expected OAuth 2 access token, login cookie or other valid authentication credential. See https://developers.google.com/identity/sign-in/web/devconsole-project.', 'status': 'UNAUTHENTICATED', 'details': [{'@type': 'type.googleapis.com/google.rpc.ErrorInfo', 'reason': 'ACCESS_TOKEN_TYPE_UNSUPPORTED', 'metadata': {'method': 'google.ai.generativelanguage.v1main.GenerativeService.GenerateContent', 'service': 'generativelanguage.googleapis.com'}}]}}]</t>
+        </is>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B201" t="inlineStr">
+        <is>
+          <t>10:53:02</t>
+        </is>
+      </c>
+      <c r="C201" t="inlineStr">
+        <is>
+          <t>2100175569618948352</t>
+        </is>
+      </c>
+      <c r="D201" t="inlineStr">
+        <is>
+          <t>LcioLaboissier2</t>
+        </is>
+      </c>
+      <c r="E201" t="inlineStr">
+        <is>
+          <t>@vamosdireita É jogo de marketing podre.</t>
+        </is>
+      </c>
+      <c r="F201" t="inlineStr">
+        <is>
+          <t>https://x.com/LcioLaboissier2/status/2100175569618948352</t>
+        </is>
+      </c>
+      <c r="H201" t="n">
+        <v>0</v>
+      </c>
+      <c r="I201" t="n">
+        <v>0</v>
+      </c>
+      <c r="J201" t="inlineStr">
+        <is>
+          <t>multi_group</t>
+        </is>
+      </c>
+      <c r="L201" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="N201" t="inlineStr">
+        <is>
+          <t>Error code: 401 - [{'error': {'code': 401, 'message': 'Request had invalid authentication credentials. Expected OAuth 2 access token, login cookie or other valid authentication credential. See https://developers.google.com/identity/sign-in/web/devconsole-project.', 'status': 'UNAUTHENTICATED', 'details': [{'@type': 'type.googleapis.com/google.rpc.ErrorInfo', 'reason': 'ACCESS_TOKEN_TYPE_UNSUPPORTED', 'metadata': {'method': 'google.ai.generativelanguage.v1main.GenerativeService.GenerateContent', 'service': 'generativelanguage.googleapis.com'}}]}}]</t>
+        </is>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B202" t="inlineStr">
+        <is>
+          <t>10:53:02</t>
+        </is>
+      </c>
+      <c r="C202" t="inlineStr">
+        <is>
+          <t>2100175568960458903</t>
+        </is>
+      </c>
+      <c r="D202" t="inlineStr">
+        <is>
+          <t>SamueleOnelia</t>
+        </is>
+      </c>
+      <c r="E202" t="inlineStr">
+        <is>
+          <t>@diodo_e If your goal is to attract creators or aspiring creators, sharing MRR is a proven marketing tactic.</t>
+        </is>
+      </c>
+      <c r="F202" t="inlineStr">
+        <is>
+          <t>https://x.com/SamueleOnelia/status/2100175568960458903</t>
+        </is>
+      </c>
+      <c r="H202" t="n">
+        <v>0</v>
+      </c>
+      <c r="I202" t="n">
+        <v>0</v>
+      </c>
+      <c r="J202" t="inlineStr">
+        <is>
+          <t>multi_group</t>
+        </is>
+      </c>
+      <c r="L202" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="N202" t="inlineStr">
+        <is>
+          <t>Error code: 401 - [{'error': {'code': 401, 'message': 'Request had invalid authentication credentials. Expected OAuth 2 access token, login cookie or other valid authentication credential. See https://developers.google.com/identity/sign-in/web/devconsole-project.', 'status': 'UNAUTHENTICATED', 'details': [{'@type': 'type.googleapis.com/google.rpc.ErrorInfo', 'reason': 'ACCESS_TOKEN_TYPE_UNSUPPORTED', 'metadata': {'method': 'google.ai.generativelanguage.v1main.GenerativeService.GenerateContent', 'service': 'generativelanguage.googleapis.com'}}]}}]</t>
+        </is>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B203" t="inlineStr">
+        <is>
+          <t>10:53:02</t>
+        </is>
+      </c>
+      <c r="C203" t="inlineStr">
+        <is>
+          <t>2100175558370078727</t>
+        </is>
+      </c>
+      <c r="D203" t="inlineStr">
+        <is>
+          <t>s_ketharaman</t>
+        </is>
+      </c>
+      <c r="E203" t="inlineStr">
+        <is>
+          <t>"When OpenAI goes public, I assume it will need to claim a 15% probability of killing everyone." ~ @matt_levine.
+Never struck me in my whole life of doing B2B Tech Marketing that I should've focused on risk factors instead of wasting time on features, benefits, etc. 😀. https://t.co/ZM8wT7zqUY</t>
+        </is>
+      </c>
+      <c r="F203" t="inlineStr">
+        <is>
+          <t>https://x.com/s_ketharaman/status/2100175558370078727</t>
+        </is>
+      </c>
+      <c r="H203" t="n">
+        <v>0</v>
+      </c>
+      <c r="I203" t="n">
+        <v>0</v>
+      </c>
+      <c r="J203" t="inlineStr">
+        <is>
+          <t>multi_group</t>
+        </is>
+      </c>
+      <c r="L203" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="N203" t="inlineStr">
+        <is>
+          <t>Error code: 401 - [{'error': {'code': 401, 'message': 'Request had invalid authentication credentials. Expected OAuth 2 access token, login cookie or other valid authentication credential. See https://developers.google.com/identity/sign-in/web/devconsole-project.', 'status': 'UNAUTHENTICATED', 'details': [{'@type': 'type.googleapis.com/google.rpc.ErrorInfo', 'reason': 'ACCESS_TOKEN_TYPE_UNSUPPORTED', 'metadata': {'method': 'google.ai.generativelanguage.v1main.GenerativeService.GenerateContent', 'service': 'generativelanguage.googleapis.com'}}]}}]</t>
+        </is>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B204" t="inlineStr">
+        <is>
+          <t>10:53:02</t>
+        </is>
+      </c>
+      <c r="C204" t="inlineStr">
+        <is>
+          <t>2100175553013985399</t>
+        </is>
+      </c>
+      <c r="D204" t="inlineStr">
+        <is>
+          <t>VengefulFrieren</t>
+        </is>
+      </c>
+      <c r="E204" t="inlineStr">
+        <is>
+          <t>@Alisa_KujouLARP His father works in marketing.
+"it's over, this will be the last video" and then a few minutes later he suggest his son might make new videos soon. https://t.co/8zq6UJJqc3</t>
+        </is>
+      </c>
+      <c r="F204" t="inlineStr">
+        <is>
+          <t>https://x.com/VengefulFrieren/status/2100175553013985399</t>
+        </is>
+      </c>
+      <c r="H204" t="n">
+        <v>0</v>
+      </c>
+      <c r="I204" t="n">
+        <v>0</v>
+      </c>
+      <c r="J204" t="inlineStr">
+        <is>
+          <t>multi_group</t>
+        </is>
+      </c>
+      <c r="L204" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="N204" t="inlineStr">
+        <is>
+          <t>Error code: 401 - [{'error': {'code': 401, 'message': 'Request had invalid authentication credentials. Expected OAuth 2 access token, login cookie or other valid authentication credential. See https://developers.google.com/identity/sign-in/web/devconsole-project.', 'status': 'UNAUTHENTICATED', 'details': [{'@type': 'type.googleapis.com/google.rpc.ErrorInfo', 'reason': 'ACCESS_TOKEN_TYPE_UNSUPPORTED', 'metadata': {'method': 'google.ai.generativelanguage.v1main.GenerativeService.GenerateContent', 'service': 'generativelanguage.googleapis.com'}}]}}]</t>
+        </is>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B205" t="inlineStr">
+        <is>
+          <t>10:53:02</t>
+        </is>
+      </c>
+      <c r="C205" t="inlineStr">
+        <is>
+          <t>2100175528473034773</t>
+        </is>
+      </c>
+      <c r="D205" t="inlineStr">
+        <is>
+          <t>jakeh2792</t>
+        </is>
+      </c>
+      <c r="E205" t="inlineStr">
+        <is>
+          <t>China won’t will the LLM race, but is winning the robotics race. 
+One is marketing centric, the other product centric. 
+China struggles to do brand, US struggles with creating mass market hardware.</t>
+        </is>
+      </c>
+      <c r="F205" t="inlineStr">
+        <is>
+          <t>https://x.com/jakeh2792/status/2100175528473034773</t>
+        </is>
+      </c>
+      <c r="H205" t="n">
+        <v>0</v>
+      </c>
+      <c r="I205" t="n">
+        <v>0</v>
+      </c>
+      <c r="J205" t="inlineStr">
+        <is>
+          <t>multi_group</t>
+        </is>
+      </c>
+      <c r="L205" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="N205" t="inlineStr">
+        <is>
+          <t>Error code: 401 - [{'error': {'code': 401, 'message': 'Request had invalid authentication credentials. Expected OAuth 2 access token, login cookie or other valid authentication credential. See https://developers.google.com/identity/sign-in/web/devconsole-project.', 'status': 'UNAUTHENTICATED', 'details': [{'@type': 'type.googleapis.com/google.rpc.ErrorInfo', 'reason': 'ACCESS_TOKEN_TYPE_UNSUPPORTED', 'metadata': {'service': 'generativelanguage.googleapis.com', 'method': 'google.ai.generativelanguage.v1main.GenerativeService.GenerateContent'}}]}}]</t>
+        </is>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B206" t="inlineStr">
+        <is>
+          <t>10:53:02</t>
+        </is>
+      </c>
+      <c r="C206" t="inlineStr">
+        <is>
+          <t>2100175484529360932</t>
+        </is>
+      </c>
+      <c r="D206" t="inlineStr">
+        <is>
+          <t>zmb_bllbry_mffn</t>
+        </is>
+      </c>
+      <c r="E206" t="inlineStr">
+        <is>
+          <t>So, it is aimed at the rich class to fund services for the poor. 
+How are such low iq people able to reach the top? 
+FIRE YOUR MARKETING TEAM</t>
+        </is>
+      </c>
+      <c r="F206" t="inlineStr">
+        <is>
+          <t>https://x.com/zmb_bllbry_mffn/status/2100175484529360932</t>
+        </is>
+      </c>
+      <c r="H206" t="n">
+        <v>0</v>
+      </c>
+      <c r="I206" t="n">
+        <v>0</v>
+      </c>
+      <c r="J206" t="inlineStr">
+        <is>
+          <t>multi_group</t>
+        </is>
+      </c>
+      <c r="L206" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="N206" t="inlineStr">
+        <is>
+          <t>Error code: 401 - [{'error': {'code': 401, 'message': 'Request had invalid authentication credentials. Expected OAuth 2 access token, login cookie or other valid authentication credential. See https://developers.google.com/identity/sign-in/web/devconsole-project.', 'status': 'UNAUTHENTICATED', 'details': [{'@type': 'type.googleapis.com/google.rpc.ErrorInfo', 'reason': 'ACCESS_TOKEN_TYPE_UNSUPPORTED', 'metadata': {'method': 'google.ai.generativelanguage.v1main.GenerativeService.GenerateContent', 'service': 'generativelanguage.googleapis.com'}}]}}]</t>
+        </is>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B207" t="inlineStr">
+        <is>
+          <t>10:53:02</t>
+        </is>
+      </c>
+      <c r="C207" t="inlineStr">
+        <is>
+          <t>2100175480033059081</t>
+        </is>
+      </c>
+      <c r="D207" t="inlineStr">
+        <is>
+          <t>obito12OG</t>
+        </is>
+      </c>
+      <c r="E207" t="inlineStr">
+        <is>
+          <t>@CoderJunkie Trust the math, not the marketing page.</t>
+        </is>
+      </c>
+      <c r="F207" t="inlineStr">
+        <is>
+          <t>https://x.com/obito12OG/status/2100175480033059081</t>
+        </is>
+      </c>
+      <c r="H207" t="n">
+        <v>0</v>
+      </c>
+      <c r="I207" t="n">
+        <v>0</v>
+      </c>
+      <c r="J207" t="inlineStr">
+        <is>
+          <t>multi_group</t>
+        </is>
+      </c>
+      <c r="L207" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="N207" t="inlineStr">
+        <is>
+          <t>Error code: 401 - [{'error': {'code': 401, 'message': 'Request had invalid authentication credentials. Expected OAuth 2 access token, login cookie or other valid authentication credential. See https://developers.google.com/identity/sign-in/web/devconsole-project.', 'status': 'UNAUTHENTICATED', 'details': [{'@type': 'type.googleapis.com/google.rpc.ErrorInfo', 'reason': 'ACCESS_TOKEN_TYPE_UNSUPPORTED', 'metadata': {'method': 'google.ai.generativelanguage.v1main.GenerativeService.GenerateContent', 'service': 'generativelanguage.googleapis.com'}}]}}]</t>
+        </is>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B208" t="inlineStr">
+        <is>
+          <t>10:53:02</t>
+        </is>
+      </c>
+      <c r="C208" t="inlineStr">
+        <is>
+          <t>2100175479135220026</t>
+        </is>
+      </c>
+      <c r="D208" t="inlineStr">
+        <is>
+          <t>FrankDijkstra4</t>
+        </is>
+      </c>
+      <c r="E208" t="inlineStr">
+        <is>
+          <t>@VrijndeSteede @VVD Dé VVD bestaat al enige tijd niet meer. Eén pot snotterig nat met het CDA en het despotische D66. Ben al lang geleden met die visie en inhoudsloze marketing clubjes gestopt. clubjesgestopt</t>
+        </is>
+      </c>
+      <c r="F208" t="inlineStr">
+        <is>
+          <t>https://x.com/FrankDijkstra4/status/2100175479135220026</t>
+        </is>
+      </c>
+      <c r="H208" t="n">
+        <v>0</v>
+      </c>
+      <c r="I208" t="n">
+        <v>0</v>
+      </c>
+      <c r="J208" t="inlineStr">
+        <is>
+          <t>multi_group</t>
+        </is>
+      </c>
+      <c r="L208" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="N208" t="inlineStr">
+        <is>
+          <t>Error code: 401 - [{'error': {'code': 401, 'message': 'Request had invalid authentication credentials. Expected OAuth 2 access token, login cookie or other valid authentication credential. See https://developers.google.com/identity/sign-in/web/devconsole-project.', 'status': 'UNAUTHENTICATED', 'details': [{'@type': 'type.googleapis.com/google.rpc.ErrorInfo', 'reason': 'ACCESS_TOKEN_TYPE_UNSUPPORTED', 'metadata': {'service': 'generativelanguage.googleapis.com', 'method': 'google.ai.generativelanguage.v1main.GenerativeService.GenerateContent'}}]}}]</t>
+        </is>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B209" t="inlineStr">
+        <is>
+          <t>10:53:02</t>
+        </is>
+      </c>
+      <c r="C209" t="inlineStr">
+        <is>
+          <t>2100175464274739352</t>
+        </is>
+      </c>
+      <c r="D209" t="inlineStr">
+        <is>
+          <t>MarketingEdgeM</t>
+        </is>
+      </c>
+      <c r="E209" t="inlineStr">
+        <is>
+          <t>NBC marks 75 years in Nigeria! 
+Celebrating with a gala in Abuja, @CocaCola HBC reaffirmed its $1B investment plan &amp;amp; announced $2.5M in grants for youth entrepreneurs &amp;amp; clean water projects.
+Read more on our website! 
+#MarketingEdge #NBC75 #CocaColaHBC #RalphTathagata https://t.co/VPCYJrZGsS</t>
+        </is>
+      </c>
+      <c r="F209" t="inlineStr">
+        <is>
+          <t>https://x.com/MarketingEdgeM/status/2100175464274739352</t>
+        </is>
+      </c>
+      <c r="H209" t="n">
+        <v>0</v>
+      </c>
+      <c r="I209" t="n">
+        <v>0</v>
+      </c>
+      <c r="J209" t="inlineStr">
+        <is>
+          <t>multi_group</t>
+        </is>
+      </c>
+      <c r="L209" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="N209" t="inlineStr">
+        <is>
+          <t>Error code: 401 - [{'error': {'code': 401, 'message': 'Request had invalid authentication credentials. Expected OAuth 2 access token, login cookie or other valid authentication credential. See https://developers.google.com/identity/sign-in/web/devconsole-project.', 'status': 'UNAUTHENTICATED', 'details': [{'@type': 'type.googleapis.com/google.rpc.ErrorInfo', 'reason': 'ACCESS_TOKEN_TYPE_UNSUPPORTED', 'metadata': {'method': 'google.ai.generativelanguage.v1main.GenerativeService.GenerateContent', 'service': 'generativelanguage.googleapis.com'}}]}}]</t>
+        </is>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B210" t="inlineStr">
+        <is>
+          <t>10:53:02</t>
+        </is>
+      </c>
+      <c r="C210" t="inlineStr">
+        <is>
+          <t>2100175464728056136</t>
+        </is>
+      </c>
+      <c r="D210" t="inlineStr">
+        <is>
+          <t>GfxRabbi</t>
+        </is>
+      </c>
+      <c r="E210" t="inlineStr">
+        <is>
+          <t>Small Streamer &amp;amp; Content Creator🔥📢🚀
+1.  Like ❤️
+2. Reposts🔄
+3. Comments 
+4. Drops link yt/twitch↩️
+Follow me 🔥
+Dm me for spacial promo📩🚀
+#yt
+#kick
+#twitch
+#youtube
+#gaming
+#smallstreamer 
+#contentcreator 
+#SmallBusiness 
+#promotion https://t.co/n0iJMV7RDj</t>
+        </is>
+      </c>
+      <c r="F210" t="inlineStr">
+        <is>
+          <t>https://x.com/GfxRabbi/status/2100175464728056136</t>
+        </is>
+      </c>
+      <c r="H210" t="n">
+        <v>0</v>
+      </c>
+      <c r="I210" t="n">
+        <v>0</v>
+      </c>
+      <c r="J210" t="inlineStr">
+        <is>
+          <t>multi_group</t>
+        </is>
+      </c>
+      <c r="L210" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="N210" t="inlineStr">
+        <is>
+          <t>Error code: 401 - [{'error': {'code': 401, 'message': 'Request had invalid authentication credentials. Expected OAuth 2 access token, login cookie or other valid authentication credential. See https://developers.google.com/identity/sign-in/web/devconsole-project.', 'status': 'UNAUTHENTICATED', 'details': [{'@type': 'type.googleapis.com/google.rpc.ErrorInfo', 'reason': 'ACCESS_TOKEN_TYPE_UNSUPPORTED', 'metadata': {'method': 'google.ai.generativelanguage.v1main.GenerativeService.GenerateContent', 'service': 'generativelanguage.googleapis.com'}}]}}]</t>
+        </is>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B211" t="inlineStr">
+        <is>
+          <t>10:53:02</t>
+        </is>
+      </c>
+      <c r="C211" t="inlineStr">
+        <is>
+          <t>2100176053604102383</t>
+        </is>
+      </c>
+      <c r="D211" t="inlineStr">
+        <is>
+          <t>GfxRabbi</t>
+        </is>
+      </c>
+      <c r="E211" t="inlineStr">
+        <is>
+          <t>🚀Small streamer &amp;amp; content creator need growth?
+Build your YouTube,Twitch &amp;amp; Kick streams NOW!
+Drop links below✅
+Like❤️Comment💬Repost🔄
+DM me for spacial promo &amp;amp; exclusive  growth!🚀
+#Twitch #TwitchStreamer #Kick #Gaming #SmallStreamer #ContentCreator #YouTubeGrowth https://t.co/RFSRlRWFFK</t>
+        </is>
+      </c>
+      <c r="F211" t="inlineStr">
+        <is>
+          <t>https://x.com/GfxRabbi/status/2100176053604102383</t>
+        </is>
+      </c>
+      <c r="H211" t="n">
+        <v>0</v>
+      </c>
+      <c r="I211" t="n">
+        <v>0</v>
+      </c>
+      <c r="J211" t="inlineStr">
+        <is>
+          <t>multi_group</t>
+        </is>
+      </c>
+      <c r="L211" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="N211" t="inlineStr">
+        <is>
+          <t>Error code: 401 - [{'error': {'code': 401, 'message': 'Request had invalid authentication credentials. Expected OAuth 2 access token, login cookie or other valid authentication credential. See https://developers.google.com/identity/sign-in/web/devconsole-project.', 'status': 'UNAUTHENTICATED', 'details': [{'@type': 'type.googleapis.com/google.rpc.ErrorInfo', 'reason': 'ACCESS_TOKEN_TYPE_UNSUPPORTED', 'metadata': {'service': 'generativelanguage.googleapis.com', 'method': 'google.ai.generativelanguage.v1main.GenerativeService.GenerateContent'}}]}}]</t>
+        </is>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B212" t="inlineStr">
+        <is>
+          <t>10:53:03</t>
+        </is>
+      </c>
+      <c r="C212" t="inlineStr">
+        <is>
+          <t>2100175361833394371</t>
+        </is>
+      </c>
+      <c r="D212" t="inlineStr">
+        <is>
+          <t>iRubankt</t>
+        </is>
+      </c>
+      <c r="E212" t="inlineStr">
+        <is>
+          <t>Google Ads AI needs guardrails, not blind trust ft Mike Ryan
+https://t.co/n9MN4g2CLo</t>
+        </is>
+      </c>
+      <c r="F212" t="inlineStr">
+        <is>
+          <t>https://x.com/iRubankt/status/2100175361833394371</t>
+        </is>
+      </c>
+      <c r="H212" t="n">
+        <v>0</v>
+      </c>
+      <c r="I212" t="n">
+        <v>0</v>
+      </c>
+      <c r="J212" t="inlineStr">
+        <is>
+          <t>multi_group</t>
+        </is>
+      </c>
+      <c r="L212" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="N212" t="inlineStr">
+        <is>
+          <t>Error code: 401 - [{'error': {'code': 401, 'message': 'Request had invalid authentication credentials. Expected OAuth 2 access token, login cookie or other valid authentication credential. See https://developers.google.com/identity/sign-in/web/devconsole-project.', 'status': 'UNAUTHENTICATED', 'details': [{'@type': 'type.googleapis.com/google.rpc.ErrorInfo', 'reason': 'ACCESS_TOKEN_TYPE_UNSUPPORTED', 'metadata': {'method': 'google.ai.generativelanguage.v1main.GenerativeService.GenerateContent', 'service': 'generativelanguage.googleapis.com'}}]}}]</t>
+        </is>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B213" t="inlineStr">
+        <is>
+          <t>10:53:03</t>
+        </is>
+      </c>
+      <c r="C213" t="inlineStr">
+        <is>
+          <t>2100175974205682167</t>
+        </is>
+      </c>
+      <c r="D213" t="inlineStr">
+        <is>
+          <t>RolandAsare_</t>
+        </is>
+      </c>
+      <c r="E213" t="inlineStr">
+        <is>
+          <t>GOD’S WORK AT NSAWAM
+Sometimes, transformation begins in places where society least expects it.
+At Nsawam Prison, a remarkable reform initiative is giving inmates something more valuable than punishment alone: a second chance at life.
+Through an educational and rehabilitation</t>
+        </is>
+      </c>
+      <c r="F213" t="inlineStr">
+        <is>
+          <t>https://x.com/RolandAsare_/status/2100175974205682167</t>
+        </is>
+      </c>
+      <c r="H213" t="n">
+        <v>0</v>
+      </c>
+      <c r="I213" t="n">
+        <v>0</v>
+      </c>
+      <c r="J213" t="inlineStr">
+        <is>
+          <t>multi_group</t>
+        </is>
+      </c>
+      <c r="L213" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="N213" t="inlineStr">
+        <is>
+          <t>Error code: 401 - [{'error': {'code': 401, 'message': 'Request had invalid authentication credentials. Expected OAuth 2 access token, login cookie or other valid authentication credential. See https://developers.google.com/identity/sign-in/web/devconsole-project.', 'status': 'UNAUTHENTICATED', 'details': [{'@type': 'type.googleapis.com/google.rpc.ErrorInfo', 'reason': 'ACCESS_TOKEN_TYPE_UNSUPPORTED', 'metadata': {'method': 'google.ai.generativelanguage.v1main.GenerativeService.GenerateContent', 'service': 'generativelanguage.googleapis.com'}}]}}]</t>
+        </is>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B214" t="inlineStr">
+        <is>
+          <t>10:53:03</t>
+        </is>
+      </c>
+      <c r="C214" t="inlineStr">
+        <is>
+          <t>2100175945055301952</t>
+        </is>
+      </c>
+      <c r="D214" t="inlineStr">
+        <is>
+          <t>freelancewizzy</t>
+        </is>
+      </c>
+      <c r="E214" t="inlineStr">
+        <is>
+          <t>@bluenokii // yeah that's basically my thoughts exactly, I mean I'm the oldest out of the three in my family so I can sorta take care of them but I don't think I'd be a good parent at all 😭😭 I don't want to hurt them by accident</t>
+        </is>
+      </c>
+      <c r="F214" t="inlineStr">
+        <is>
+          <t>https://x.com/freelancewizzy/status/2100175945055301952</t>
+        </is>
+      </c>
+      <c r="H214" t="n">
+        <v>0</v>
+      </c>
+      <c r="I214" t="n">
+        <v>0</v>
+      </c>
+      <c r="J214" t="inlineStr">
+        <is>
+          <t>multi_group</t>
+        </is>
+      </c>
+      <c r="L214" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="N214" t="inlineStr">
+        <is>
+          <t>Error code: 401 - [{'error': {'code': 401, 'message': 'Request had invalid authentication credentials. Expected OAuth 2 access token, login cookie or other valid authentication credential. See https://developers.google.com/identity/sign-in/web/devconsole-project.', 'status': 'UNAUTHENTICATED', 'details': [{'@type': 'type.googleapis.com/google.rpc.ErrorInfo', 'reason': 'ACCESS_TOKEN_TYPE_UNSUPPORTED', 'metadata': {'method': 'google.ai.generativelanguage.v1main.GenerativeService.GenerateContent', 'service': 'generativelanguage.googleapis.com'}}]}}]</t>
+        </is>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B215" t="inlineStr">
+        <is>
+          <t>10:53:03</t>
+        </is>
+      </c>
+      <c r="C215" t="inlineStr">
+        <is>
+          <t>2100175942723215680</t>
+        </is>
+      </c>
+      <c r="D215" t="inlineStr">
+        <is>
+          <t>KIZO_ES</t>
+        </is>
+      </c>
+      <c r="E215" t="inlineStr">
+        <is>
+          <t>@Riley_Ikni you might remember, you one roasted my landing page and gave me encouragement to keep building  Tusk. It's now released for some time and slowly growing:
+https://t.co/k8LK9uXr9P</t>
+        </is>
+      </c>
+      <c r="F215" t="inlineStr">
+        <is>
+          <t>https://x.com/KIZO_ES/status/2100175942723215680</t>
+        </is>
+      </c>
+      <c r="H215" t="n">
+        <v>0</v>
+      </c>
+      <c r="I215" t="n">
+        <v>0</v>
+      </c>
+      <c r="J215" t="inlineStr">
+        <is>
+          <t>multi_group</t>
+        </is>
+      </c>
+      <c r="L215" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="N215" t="inlineStr">
+        <is>
+          <t>Error code: 401 - [{'error': {'code': 401, 'message': 'Request had invalid authentication credentials. Expected OAuth 2 access token, login cookie or other valid authentication credential. See https://developers.google.com/identity/sign-in/web/devconsole-project.', 'status': 'UNAUTHENTICATED', 'details': [{'@type': 'type.googleapis.com/google.rpc.ErrorInfo', 'reason': 'ACCESS_TOKEN_TYPE_UNSUPPORTED', 'metadata': {'method': 'google.ai.generativelanguage.v1main.GenerativeService.GenerateContent', 'service': 'generativelanguage.googleapis.com'}}]}}]</t>
+        </is>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B216" t="inlineStr">
+        <is>
+          <t>10:53:03</t>
+        </is>
+      </c>
+      <c r="C216" t="inlineStr">
+        <is>
+          <t>2100175920724132042</t>
+        </is>
+      </c>
+      <c r="D216" t="inlineStr">
+        <is>
+          <t>GrownixApp</t>
+        </is>
+      </c>
+      <c r="E216" t="inlineStr">
+        <is>
+          <t>Day 3 of posting TikTok slideshows.
+I usually create the slideshow first thing in the morning. That seems to be my best window for creativity.
+This time I found a viral post from a completely different niche and rebuilt the idea for ours.
+No CTA this time.
+I already had a</t>
+        </is>
+      </c>
+      <c r="F216" t="inlineStr">
+        <is>
+          <t>https://x.com/GrownixApp/status/2100175920724132042</t>
+        </is>
+      </c>
+      <c r="H216" t="n">
+        <v>0</v>
+      </c>
+      <c r="I216" t="n">
+        <v>0</v>
+      </c>
+      <c r="J216" t="inlineStr">
+        <is>
+          <t>multi_group</t>
+        </is>
+      </c>
+      <c r="L216" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="N216" t="inlineStr">
+        <is>
+          <t>Error code: 401 - [{'error': {'code': 401, 'message': 'Request had invalid authentication credentials. Expected OAuth 2 access token, login cookie or other valid authentication credential. See https://developers.google.com/identity/sign-in/web/devconsole-project.', 'status': 'UNAUTHENTICATED', 'details': [{'@type': 'type.googleapis.com/google.rpc.ErrorInfo', 'reason': 'ACCESS_TOKEN_TYPE_UNSUPPORTED', 'metadata': {'service': 'generativelanguage.googleapis.com', 'method': 'google.ai.generativelanguage.v1main.GenerativeService.GenerateContent'}}]}}]</t>
+        </is>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B217" t="inlineStr">
+        <is>
+          <t>10:53:03</t>
+        </is>
+      </c>
+      <c r="C217" t="inlineStr">
+        <is>
+          <t>2100175915460260273</t>
+        </is>
+      </c>
+      <c r="D217" t="inlineStr">
+        <is>
+          <t>williamdtc2y</t>
+        </is>
+      </c>
+      <c r="E217" t="inlineStr">
+        <is>
+          <t>@zerdotre I have message you</t>
+        </is>
+      </c>
+      <c r="F217" t="inlineStr">
+        <is>
+          <t>https://x.com/williamdtc2y/status/2100175915460260273</t>
+        </is>
+      </c>
+      <c r="H217" t="n">
+        <v>0</v>
+      </c>
+      <c r="I217" t="n">
+        <v>0</v>
+      </c>
+      <c r="J217" t="inlineStr">
+        <is>
+          <t>multi_group</t>
+        </is>
+      </c>
+      <c r="L217" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="N217" t="inlineStr">
+        <is>
+          <t>Error code: 401 - [{'error': {'code': 401, 'message': 'Request had invalid authentication credentials. Expected OAuth 2 access token, login cookie or other valid authentication credential. See https://developers.google.com/identity/sign-in/web/devconsole-project.', 'status': 'UNAUTHENTICATED', 'details': [{'@type': 'type.googleapis.com/google.rpc.ErrorInfo', 'reason': 'ACCESS_TOKEN_TYPE_UNSUPPORTED', 'metadata': {'service': 'generativelanguage.googleapis.com', 'method': 'google.ai.generativelanguage.v1main.GenerativeService.GenerateContent'}}]}}]</t>
+        </is>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B218" t="inlineStr">
+        <is>
+          <t>10:53:03</t>
+        </is>
+      </c>
+      <c r="C218" t="inlineStr">
+        <is>
+          <t>2100175906467991869</t>
+        </is>
+      </c>
+      <c r="D218" t="inlineStr">
+        <is>
+          <t>Kishan_Devani_</t>
+        </is>
+      </c>
+      <c r="E218" t="inlineStr">
+        <is>
+          <t>@vibeonX69 A better question gets a better answer. that's the whole mechanism</t>
+        </is>
+      </c>
+      <c r="F218" t="inlineStr">
+        <is>
+          <t>https://x.com/Kishan_Devani_/status/2100175906467991869</t>
+        </is>
+      </c>
+      <c r="H218" t="n">
+        <v>0</v>
+      </c>
+      <c r="I218" t="n">
+        <v>0</v>
+      </c>
+      <c r="J218" t="inlineStr">
+        <is>
+          <t>multi_group</t>
+        </is>
+      </c>
+      <c r="L218" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="N218" t="inlineStr">
+        <is>
+          <t>Error code: 401 - [{'error': {'code': 401, 'message': 'Request had invalid authentication credentials. Expected OAuth 2 access token, login cookie or other valid authentication credential. See https://developers.google.com/identity/sign-in/web/devconsole-project.', 'status': 'UNAUTHENTICATED', 'details': [{'@type': 'type.googleapis.com/google.rpc.ErrorInfo', 'reason': 'ACCESS_TOKEN_TYPE_UNSUPPORTED', 'metadata': {'method': 'google.ai.generativelanguage.v1main.GenerativeService.GenerateContent', 'service': 'generativelanguage.googleapis.com'}}]}}]</t>
+        </is>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B219" t="inlineStr">
+        <is>
+          <t>10:53:03</t>
+        </is>
+      </c>
+      <c r="C219" t="inlineStr">
+        <is>
+          <t>2100175254463119821</t>
+        </is>
+      </c>
+      <c r="D219" t="inlineStr">
+        <is>
+          <t>Mkt4eCommerce</t>
+        </is>
+      </c>
+      <c r="E219" t="inlineStr">
+        <is>
+          <t>Gestionar #GoogleAds ya no va solo de pujas y anuncios. @Geotelecom analiza cómo suben los costes, crece la automatización y por qué estrategia, datos y coordinación entre canales pesan cada vez más en eCommerce 👇
+🔗 https://t.co/csn8oVLKVJ https://t.co/AvXaHnDVt6</t>
+        </is>
+      </c>
+      <c r="F219" t="inlineStr">
+        <is>
+          <t>https://x.com/Mkt4eCommerce/status/2100175254463119821</t>
+        </is>
+      </c>
+      <c r="H219" t="n">
+        <v>1</v>
+      </c>
+      <c r="I219" t="n">
+        <v>0</v>
+      </c>
+      <c r="J219" t="inlineStr">
+        <is>
+          <t>multi_group</t>
+        </is>
+      </c>
+      <c r="L219" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="N219" t="inlineStr">
+        <is>
+          <t>Error code: 401 - [{'error': {'code': 401, 'message': 'Request had invalid authentication credentials. Expected OAuth 2 access token, login cookie or other valid authentication credential. See https://developers.google.com/identity/sign-in/web/devconsole-project.', 'status': 'UNAUTHENTICATED', 'details': [{'@type': 'type.googleapis.com/google.rpc.ErrorInfo', 'reason': 'ACCESS_TOKEN_TYPE_UNSUPPORTED', 'metadata': {'method': 'google.ai.generativelanguage.v1main.GenerativeService.GenerateContent', 'service': 'generativelanguage.googleapis.com'}}]}}]</t>
+        </is>
+      </c>
+    </row>
+    <row r="220">
+      <c r="A220" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B220" t="inlineStr">
+        <is>
+          <t>10:53:03</t>
+        </is>
+      </c>
+      <c r="C220" t="inlineStr">
+        <is>
+          <t>2100175886200783001</t>
+        </is>
+      </c>
+      <c r="D220" t="inlineStr">
+        <is>
+          <t>emmemkay</t>
+        </is>
+      </c>
+      <c r="E220" t="inlineStr">
+        <is>
+          <t>If low self esteem and this mental slavery that women are putting themselves in did not end one woman, the rest will not learn that their body is not a machine or a glass</t>
+        </is>
+      </c>
+      <c r="F220" t="inlineStr">
+        <is>
+          <t>https://x.com/emmemkay/status/2100175886200783001</t>
+        </is>
+      </c>
+      <c r="H220" t="n">
+        <v>0</v>
+      </c>
+      <c r="I220" t="n">
+        <v>0</v>
+      </c>
+      <c r="J220" t="inlineStr">
+        <is>
+          <t>multi_group</t>
+        </is>
+      </c>
+      <c r="L220" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="N220" t="inlineStr">
+        <is>
+          <t>Error code: 401 - [{'error': {'code': 401, 'message': 'Request had invalid authentication credentials. Expected OAuth 2 access token, login cookie or other valid authentication credential. See https://developers.google.com/identity/sign-in/web/devconsole-project.', 'status': 'UNAUTHENTICATED', 'details': [{'@type': 'type.googleapis.com/google.rpc.ErrorInfo', 'reason': 'ACCESS_TOKEN_TYPE_UNSUPPORTED', 'metadata': {'method': 'google.ai.generativelanguage.v1main.GenerativeService.GenerateContent', 'service': 'generativelanguage.googleapis.com'}}]}}]</t>
+        </is>
+      </c>
+    </row>
+    <row r="221">
+      <c r="A221" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B221" t="inlineStr">
+        <is>
+          <t>10:53:03</t>
+        </is>
+      </c>
+      <c r="C221" t="inlineStr">
+        <is>
+          <t>2100175855695905063</t>
+        </is>
+      </c>
+      <c r="D221" t="inlineStr">
+        <is>
+          <t>TawohAwa</t>
+        </is>
+      </c>
+      <c r="E221" t="inlineStr">
+        <is>
+          <t>Stop telling ChatGPT “Build me a website”
+Stop telling ChatGPT “Make my website look better”
+Stop telling ChatGPT “Create a landing page”
+Bad request = Bad result.
+Use this workflow to create beautiful websites that don’t just look good  but they convert. 👇</t>
+        </is>
+      </c>
+      <c r="F221" t="inlineStr">
+        <is>
+          <t>https://x.com/TawohAwa/status/2100175855695905063</t>
+        </is>
+      </c>
+      <c r="H221" t="n">
+        <v>1</v>
+      </c>
+      <c r="I221" t="n">
+        <v>1</v>
+      </c>
+      <c r="J221" t="inlineStr">
+        <is>
+          <t>multi_group</t>
+        </is>
+      </c>
+      <c r="L221" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="N221" t="inlineStr">
+        <is>
+          <t>Error code: 401 - [{'error': {'code': 401, 'message': 'Request had invalid authentication credentials. Expected OAuth 2 access token, login cookie or other valid authentication credential. See https://developers.google.com/identity/sign-in/web/devconsole-project.', 'status': 'UNAUTHENTICATED', 'details': [{'@type': 'type.googleapis.com/google.rpc.ErrorInfo', 'reason': 'ACCESS_TOKEN_TYPE_UNSUPPORTED', 'metadata': {'method': 'google.ai.generativelanguage.v1main.GenerativeService.GenerateContent', 'service': 'generativelanguage.googleapis.com'}}]}}]</t>
+        </is>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B222" t="inlineStr">
+        <is>
+          <t>10:53:04</t>
+        </is>
+      </c>
+      <c r="C222" t="inlineStr">
+        <is>
+          <t>2100175863673504185</t>
+        </is>
+      </c>
+      <c r="D222" t="inlineStr">
+        <is>
+          <t>TawohAwa</t>
+        </is>
+      </c>
+      <c r="E222" t="inlineStr">
+        <is>
+          <t>2/ How does it work?
+Instead of asking ChatGPT to “write HTML,” ask it to build a website by selecting ‘ChatGPT work’
+Example prompt:
+Build me a modern SaaS landing page for my gym with subscriptions
+In a few minutes, ChatGPT generates a complete website preview. https://t.co/eEoSC52o8g</t>
+        </is>
+      </c>
+      <c r="F222" t="inlineStr">
+        <is>
+          <t>https://x.com/TawohAwa/status/2100175863673504185</t>
+        </is>
+      </c>
+      <c r="H222" t="n">
+        <v>0</v>
+      </c>
+      <c r="I222" t="n">
+        <v>1</v>
+      </c>
+      <c r="J222" t="inlineStr">
+        <is>
+          <t>multi_group</t>
+        </is>
+      </c>
+      <c r="L222" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="N222" t="inlineStr">
+        <is>
+          <t>Error code: 401 - [{'error': {'code': 401, 'message': 'Request had invalid authentication credentials. Expected OAuth 2 access token, login cookie or other valid authentication credential. See https://developers.google.com/identity/sign-in/web/devconsole-project.', 'status': 'UNAUTHENTICATED', 'details': [{'@type': 'type.googleapis.com/google.rpc.ErrorInfo', 'reason': 'ACCESS_TOKEN_TYPE_UNSUPPORTED', 'metadata': {'method': 'google.ai.generativelanguage.v1main.GenerativeService.GenerateContent', 'service': 'generativelanguage.googleapis.com'}}]}}]</t>
+        </is>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B223" t="inlineStr">
+        <is>
+          <t>10:53:04</t>
+        </is>
+      </c>
+      <c r="C223" t="inlineStr">
+        <is>
+          <t>2100175874817413529</t>
+        </is>
+      </c>
+      <c r="D223" t="inlineStr">
+        <is>
+          <t>KUMEYUR1</t>
+        </is>
+      </c>
+      <c r="E223" t="inlineStr">
+        <is>
+          <t>@lesbianyura SEAN THIS IS AMAZING</t>
+        </is>
+      </c>
+      <c r="F223" t="inlineStr">
+        <is>
+          <t>https://x.com/KUMEYUR1/status/2100175874817413529</t>
+        </is>
+      </c>
+      <c r="H223" t="n">
+        <v>0</v>
+      </c>
+      <c r="I223" t="n">
+        <v>0</v>
+      </c>
+      <c r="J223" t="inlineStr">
+        <is>
+          <t>multi_group</t>
+        </is>
+      </c>
+      <c r="L223" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="N223" t="inlineStr">
+        <is>
+          <t>Error code: 401 - [{'error': {'code': 401, 'message': 'Request had invalid authentication credentials. Expected OAuth 2 access token, login cookie or other valid authentication credential. See https://developers.google.com/identity/sign-in/web/devconsole-project.', 'status': 'UNAUTHENTICATED', 'details': [{'@type': 'type.googleapis.com/google.rpc.ErrorInfo', 'reason': 'ACCESS_TOKEN_TYPE_UNSUPPORTED', 'metadata': {'service': 'generativelanguage.googleapis.com', 'method': 'google.ai.generativelanguage.v1main.GenerativeService.GenerateContent'}}]}}]</t>
+        </is>
+      </c>
+    </row>
+    <row r="224">
+      <c r="A224" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B224" t="inlineStr">
+        <is>
+          <t>10:53:04</t>
+        </is>
+      </c>
+      <c r="C224" t="inlineStr">
+        <is>
+          <t>2100175858610872575</t>
+        </is>
+      </c>
+      <c r="D224" t="inlineStr">
+        <is>
+          <t>rsk9588</t>
+        </is>
+      </c>
+      <c r="E224" t="inlineStr">
+        <is>
+          <t>@annasoreskin Sure @annasoreskin</t>
+        </is>
+      </c>
+      <c r="F224" t="inlineStr">
+        <is>
+          <t>https://x.com/rsk9588/status/2100175858610872575</t>
+        </is>
+      </c>
+      <c r="H224" t="n">
+        <v>0</v>
+      </c>
+      <c r="I224" t="n">
+        <v>0</v>
+      </c>
+      <c r="J224" t="inlineStr">
+        <is>
+          <t>multi_group</t>
+        </is>
+      </c>
+      <c r="L224" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="N224" t="inlineStr">
+        <is>
+          <t>Error code: 401 - [{'error': {'code': 401, 'message': 'Request had invalid authentication credentials. Expected OAuth 2 access token, login cookie or other valid authentication credential. See https://developers.google.com/identity/sign-in/web/devconsole-project.', 'status': 'UNAUTHENTICATED', 'details': [{'@type': 'type.googleapis.com/google.rpc.ErrorInfo', 'reason': 'ACCESS_TOKEN_TYPE_UNSUPPORTED', 'metadata': {'service': 'generativelanguage.googleapis.com', 'method': 'google.ai.generativelanguage.v1main.GenerativeService.GenerateContent'}}]}}]</t>
+        </is>
+      </c>
+    </row>
+    <row r="225">
+      <c r="A225" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B225" t="inlineStr">
+        <is>
+          <t>10:53:04</t>
+        </is>
+      </c>
+      <c r="C225" t="inlineStr">
+        <is>
+          <t>2100175846162215163</t>
+        </is>
+      </c>
+      <c r="D225" t="inlineStr">
+        <is>
+          <t>ramaeeesparks</t>
+        </is>
+      </c>
+      <c r="E225" t="inlineStr">
+        <is>
+          <t>@georgeviews MoU matter illa.. Evalo convert aguthu nu pakkanum. DMK la 80 percent mela conversion rate kamichirukanga. Avanga period la convert Agatha MoU also sethu than 1 lakh crore nu kanaku kamichanga. 
+Same conversion rate or better ivanga pannrangala illa MoU mattum thana nu papom.</t>
+        </is>
+      </c>
+      <c r="F225" t="inlineStr">
+        <is>
+          <t>https://x.com/ramaeeesparks/status/2100175846162215163</t>
+        </is>
+      </c>
+      <c r="H225" t="n">
+        <v>0</v>
+      </c>
+      <c r="I225" t="n">
+        <v>0</v>
+      </c>
+      <c r="J225" t="inlineStr">
+        <is>
+          <t>multi_group</t>
+        </is>
+      </c>
+      <c r="L225" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="N225" t="inlineStr">
+        <is>
+          <t>Error code: 401 - [{'error': {'code': 401, 'message': 'Request had invalid authentication credentials. Expected OAuth 2 access token, login cookie or other valid authentication credential. See https://developers.google.com/identity/sign-in/web/devconsole-project.', 'status': 'UNAUTHENTICATED', 'details': [{'@type': 'type.googleapis.com/google.rpc.ErrorInfo', 'reason': 'ACCESS_TOKEN_TYPE_UNSUPPORTED', 'metadata': {'service': 'generativelanguage.googleapis.com', 'method': 'google.ai.generativelanguage.v1main.GenerativeService.GenerateContent'}}]}}]</t>
+        </is>
+      </c>
+    </row>
+    <row r="226">
+      <c r="A226" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B226" t="inlineStr">
+        <is>
+          <t>10:53:04</t>
+        </is>
+      </c>
+      <c r="C226" t="inlineStr">
+        <is>
+          <t>2100175836410216605</t>
+        </is>
+      </c>
+      <c r="D226" t="inlineStr">
+        <is>
+          <t>KUMEYUR1</t>
+        </is>
+      </c>
+      <c r="E226" t="inlineStr">
+        <is>
+          <t>@lesbianyura I LOVE URUHA</t>
+        </is>
+      </c>
+      <c r="F226" t="inlineStr">
+        <is>
+          <t>https://x.com/KUMEYUR1/status/2100175836410216605</t>
+        </is>
+      </c>
+      <c r="H226" t="n">
+        <v>0</v>
+      </c>
+      <c r="I226" t="n">
+        <v>0</v>
+      </c>
+      <c r="J226" t="inlineStr">
+        <is>
+          <t>multi_group</t>
+        </is>
+      </c>
+      <c r="L226" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="N226" t="inlineStr">
+        <is>
+          <t>Error code: 401 - [{'error': {'code': 401, 'message': 'Request had invalid authentication credentials. Expected OAuth 2 access token, login cookie or other valid authentication credential. See https://developers.google.com/identity/sign-in/web/devconsole-project.', 'status': 'UNAUTHENTICATED', 'details': [{'@type': 'type.googleapis.com/google.rpc.ErrorInfo', 'reason': 'ACCESS_TOKEN_TYPE_UNSUPPORTED', 'metadata': {'method': 'google.ai.generativelanguage.v1main.GenerativeService.GenerateContent', 'service': 'generativelanguage.googleapis.com'}}]}}]</t>
+        </is>
+      </c>
+    </row>
+    <row r="227">
+      <c r="A227" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B227" t="inlineStr">
+        <is>
+          <t>10:53:04</t>
+        </is>
+      </c>
+      <c r="C227" t="inlineStr">
+        <is>
+          <t>2100175807612125552</t>
+        </is>
+      </c>
+      <c r="D227" t="inlineStr">
+        <is>
+          <t>DanielKaderavek</t>
+        </is>
+      </c>
+      <c r="E227" t="inlineStr">
+        <is>
+          <t>Když to napíše liberální content creator ze @SeznamZpravy, tak to musí být pravda. Když to říká Babiš, tak to musí být nesmysl.🤦🏻‍♂️
+Jenže toto je zrovna celkem funkční řešení. Naše mladé bílé liberálky by koukaly, jak se najednou na Mostecku a Ústecku rodí děti a daň. poplatníci.</t>
+        </is>
+      </c>
+      <c r="F227" t="inlineStr">
+        <is>
+          <t>https://x.com/DanielKaderavek/status/2100175807612125552</t>
+        </is>
+      </c>
+      <c r="H227" t="n">
+        <v>1</v>
+      </c>
+      <c r="I227" t="n">
+        <v>0</v>
+      </c>
+      <c r="J227" t="inlineStr">
+        <is>
+          <t>multi_group</t>
+        </is>
+      </c>
+      <c r="L227" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="N227" t="inlineStr">
+        <is>
+          <t>Error code: 401 - [{'error': {'code': 401, 'message': 'Request had invalid authentication credentials. Expected OAuth 2 access token, login cookie or other valid authentication credential. See https://developers.google.com/identity/sign-in/web/devconsole-project.', 'status': 'UNAUTHENTICATED', 'details': [{'@type': 'type.googleapis.com/google.rpc.ErrorInfo', 'reason': 'ACCESS_TOKEN_TYPE_UNSUPPORTED', 'metadata': {'method': 'google.ai.generativelanguage.v1main.GenerativeService.GenerateContent', 'service': 'generativelanguage.googleapis.com'}}]}}]</t>
+        </is>
+      </c>
+    </row>
+    <row r="228">
+      <c r="A228" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B228" t="inlineStr">
+        <is>
+          <t>10:53:04</t>
+        </is>
+      </c>
+      <c r="C228" t="inlineStr">
+        <is>
+          <t>2100175799387144307</t>
+        </is>
+      </c>
+      <c r="D228" t="inlineStr">
+        <is>
+          <t>John_Parvu</t>
+        </is>
+      </c>
+      <c r="E228" t="inlineStr">
+        <is>
+          <t>https://t.co/UqOrCJBmD2</t>
+        </is>
+      </c>
+      <c r="F228" t="inlineStr">
+        <is>
+          <t>https://x.com/John_Parvu/status/2100175799387144307</t>
+        </is>
+      </c>
+      <c r="H228" t="n">
+        <v>0</v>
+      </c>
+      <c r="I228" t="n">
+        <v>0</v>
+      </c>
+      <c r="J228" t="inlineStr">
+        <is>
+          <t>multi_group</t>
+        </is>
+      </c>
+      <c r="L228" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="N228" t="inlineStr">
+        <is>
+          <t>Error code: 401 - [{'error': {'code': 401, 'message': 'Request had invalid authentication credentials. Expected OAuth 2 access token, login cookie or other valid authentication credential. See https://developers.google.com/identity/sign-in/web/devconsole-project.', 'status': 'UNAUTHENTICATED', 'details': [{'@type': 'type.googleapis.com/google.rpc.ErrorInfo', 'reason': 'ACCESS_TOKEN_TYPE_UNSUPPORTED', 'metadata': {'service': 'generativelanguage.googleapis.com', 'method': 'google.ai.generativelanguage.v1main.GenerativeService.GenerateContent'}}]}}]</t>
+        </is>
+      </c>
+    </row>
+    <row r="229">
+      <c r="A229" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B229" t="inlineStr">
+        <is>
+          <t>10:53:04</t>
+        </is>
+      </c>
+      <c r="C229" t="inlineStr">
+        <is>
+          <t>2100175799848497474</t>
+        </is>
+      </c>
+      <c r="D229" t="inlineStr">
+        <is>
+          <t>fakharkamario</t>
+        </is>
+      </c>
+      <c r="E229" t="inlineStr">
+        <is>
+          <t>What makes this video work:
+➜ 26 seconds. Clear structure: Hook/tease 0:00–0:05 → core message 0:05–0:10 → product demo 0:10–0:20 → outro 0:20–0:25.8. No separate problem section because the video is announcing a rebuilt product rather than introducing a new category.
+➜</t>
+        </is>
+      </c>
+      <c r="F229" t="inlineStr">
+        <is>
+          <t>https://x.com/fakharkamario/status/2100175799848497474</t>
+        </is>
+      </c>
+      <c r="H229" t="n">
+        <v>0</v>
+      </c>
+      <c r="I229" t="n">
+        <v>0</v>
+      </c>
+      <c r="J229" t="inlineStr">
+        <is>
+          <t>multi_group</t>
+        </is>
+      </c>
+      <c r="L229" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="N229" t="inlineStr">
+        <is>
+          <t>Error code: 401 - [{'error': {'code': 401, 'message': 'Request had invalid authentication credentials. Expected OAuth 2 access token, login cookie or other valid authentication credential. See https://developers.google.com/identity/sign-in/web/devconsole-project.', 'status': 'UNAUTHENTICATED', 'details': [{'@type': 'type.googleapis.com/google.rpc.ErrorInfo', 'reason': 'ACCESS_TOKEN_TYPE_UNSUPPORTED', 'metadata': {'method': 'google.ai.generativelanguage.v1main.GenerativeService.GenerateContent', 'service': 'generativelanguage.googleapis.com'}}]}}]</t>
+        </is>
+      </c>
+    </row>
+    <row r="230">
+      <c r="A230" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B230" t="inlineStr">
+        <is>
+          <t>10:53:04</t>
+        </is>
+      </c>
+      <c r="C230" t="inlineStr">
+        <is>
+          <t>2100175765216039106</t>
+        </is>
+      </c>
+      <c r="D230" t="inlineStr">
+        <is>
+          <t>marcommnews</t>
+        </is>
+      </c>
+      <c r="E230" t="inlineStr">
+        <is>
+          <t>AB Tasty and VWO unite as @wingify  to launch Agentic Experience Optimisation platform https://t.co/tbMdZVv5gs #AdTech #MarCommNews https://t.co/t2GnOWQyVL</t>
+        </is>
+      </c>
+      <c r="F230" t="inlineStr">
+        <is>
+          <t>https://x.com/marcommnews/status/2100175765216039106</t>
+        </is>
+      </c>
+      <c r="H230" t="n">
+        <v>0</v>
+      </c>
+      <c r="I230" t="n">
+        <v>0</v>
+      </c>
+      <c r="J230" t="inlineStr">
+        <is>
+          <t>multi_group</t>
+        </is>
+      </c>
+      <c r="L230" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="N230" t="inlineStr">
+        <is>
+          <t>Error code: 401 - [{'error': {'code': 401, 'message': 'Request had invalid authentication credentials. Expected OAuth 2 access token, login cookie or other valid authentication credential. See https://developers.google.com/identity/sign-in/web/devconsole-project.', 'status': 'UNAUTHENTICATED', 'details': [{'@type': 'type.googleapis.com/google.rpc.ErrorInfo', 'reason': 'ACCESS_TOKEN_TYPE_UNSUPPORTED', 'metadata': {'method': 'google.ai.generativelanguage.v1main.GenerativeService.GenerateContent', 'service': 'generativelanguage.googleapis.com'}}]}}]</t>
+        </is>
+      </c>
+    </row>
+    <row r="231">
+      <c r="A231" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B231" t="inlineStr">
+        <is>
+          <t>10:53:05</t>
+        </is>
+      </c>
+      <c r="C231" t="inlineStr">
+        <is>
+          <t>2100175755510485196</t>
+        </is>
+      </c>
+      <c r="D231" t="inlineStr">
+        <is>
+          <t>theappbulletin</t>
+        </is>
+      </c>
+      <c r="E231" t="inlineStr">
+        <is>
+          <t>@MrBrjan Who cares about originality,one shot an app,and market it better than them. Thats it</t>
+        </is>
+      </c>
+      <c r="F231" t="inlineStr">
+        <is>
+          <t>https://x.com/theappbulletin/status/2100175755510485196</t>
+        </is>
+      </c>
+      <c r="H231" t="n">
+        <v>0</v>
+      </c>
+      <c r="I231" t="n">
+        <v>0</v>
+      </c>
+      <c r="J231" t="inlineStr">
+        <is>
+          <t>multi_group</t>
+        </is>
+      </c>
+      <c r="L231" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="N231" t="inlineStr">
+        <is>
+          <t>Error code: 401 - [{'error': {'code': 401, 'message': 'Request had invalid authentication credentials. Expected OAuth 2 access token, login cookie or other valid authentication credential. See https://developers.google.com/identity/sign-in/web/devconsole-project.', 'status': 'UNAUTHENTICATED', 'details': [{'@type': 'type.googleapis.com/google.rpc.ErrorInfo', 'reason': 'ACCESS_TOKEN_TYPE_UNSUPPORTED', 'metadata': {'method': 'google.ai.generativelanguage.v1main.GenerativeService.GenerateContent', 'service': 'generativelanguage.googleapis.com'}}]}}]</t>
+        </is>
+      </c>
+    </row>
+    <row r="232">
+      <c r="A232" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B232" t="inlineStr">
+        <is>
+          <t>10:53:05</t>
+        </is>
+      </c>
+      <c r="C232" t="inlineStr">
+        <is>
+          <t>2100175749114163219</t>
+        </is>
+      </c>
+      <c r="D232" t="inlineStr">
+        <is>
+          <t>realibdouglas</t>
+        </is>
+      </c>
+      <c r="E232" t="inlineStr">
+        <is>
+          <t>@AlexTudun Happy Birthday! 🎉🍾</t>
+        </is>
+      </c>
+      <c r="F232" t="inlineStr">
+        <is>
+          <t>https://x.com/realibdouglas/status/2100175749114163219</t>
+        </is>
+      </c>
+      <c r="H232" t="n">
+        <v>0</v>
+      </c>
+      <c r="I232" t="n">
+        <v>0</v>
+      </c>
+      <c r="J232" t="inlineStr">
+        <is>
+          <t>multi_group</t>
+        </is>
+      </c>
+      <c r="L232" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="N232" t="inlineStr">
+        <is>
+          <t>Error code: 401 - [{'error': {'code': 401, 'message': 'Request had invalid authentication credentials. Expected OAuth 2 access token, login cookie or other valid authentication credential. See https://developers.google.com/identity/sign-in/web/devconsole-project.', 'status': 'UNAUTHENTICATED', 'details': [{'@type': 'type.googleapis.com/google.rpc.ErrorInfo', 'reason': 'ACCESS_TOKEN_TYPE_UNSUPPORTED', 'metadata': {'service': 'generativelanguage.googleapis.com', 'method': 'google.ai.generativelanguage.v1main.GenerativeService.GenerateContent'}}]}}]</t>
+        </is>
+      </c>
+    </row>
+    <row r="233">
+      <c r="A233" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B233" t="inlineStr">
+        <is>
+          <t>10:53:05</t>
+        </is>
+      </c>
+      <c r="C233" t="inlineStr">
+        <is>
+          <t>2100175749886124350</t>
+        </is>
+      </c>
+      <c r="D233" t="inlineStr">
+        <is>
+          <t>takumiautowork</t>
+        </is>
+      </c>
+      <c r="E233" t="inlineStr">
+        <is>
+          <t>フォロワー0人でも「今まさに商品を買おうとしてる人」を集める方法はあります。
+例えば「○○英会話 口コミ」ってGoogleで検索する人。もうそのサービスを知ってて、申し込むか迷ってる可能性あるよね。
+だったら、その人の検索結果に自分の記事を広告で出せばいい。</t>
+        </is>
+      </c>
+      <c r="F233" t="inlineStr">
+        <is>
+          <t>https://x.com/takumiautowork/status/2100175749886124350</t>
+        </is>
+      </c>
+      <c r="H233" t="n">
+        <v>0</v>
+      </c>
+      <c r="I233" t="n">
+        <v>0</v>
+      </c>
+      <c r="J233" t="inlineStr">
+        <is>
+          <t>multi_group</t>
+        </is>
+      </c>
+      <c r="L233" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="N233" t="inlineStr">
+        <is>
+          <t>Error code: 401 - [{'error': {'code': 401, 'message': 'Request had invalid authentication credentials. Expected OAuth 2 access token, login cookie or other valid authentication credential. See https://developers.google.com/identity/sign-in/web/devconsole-project.', 'status': 'UNAUTHENTICATED', 'details': [{'@type': 'type.googleapis.com/google.rpc.ErrorInfo', 'reason': 'ACCESS_TOKEN_TYPE_UNSUPPORTED', 'metadata': {'service': 'generativelanguage.googleapis.com', 'method': 'google.ai.generativelanguage.v1main.GenerativeService.GenerateContent'}}]}}]</t>
+        </is>
+      </c>
+    </row>
+    <row r="234">
+      <c r="A234" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B234" t="inlineStr">
+        <is>
+          <t>10:53:05</t>
+        </is>
+      </c>
+      <c r="C234" t="inlineStr">
+        <is>
+          <t>2100175726532039153</t>
+        </is>
+      </c>
+      <c r="D234" t="inlineStr">
+        <is>
+          <t>ayewatchai</t>
+        </is>
+      </c>
+      <c r="E234" t="inlineStr">
+        <is>
+          <t>https://t.co/AKuFrXz3EW rewrote a plan cell at 2:14am. if you had AyeWatch watching that public pricing page, it would have pinged you before slack turned into “wait, did they always include that?” @ayewatchai https://t.co/TwWgpzGmhY</t>
+        </is>
+      </c>
+      <c r="F234" t="inlineStr">
+        <is>
+          <t>https://x.com/ayewatchai/status/2100175726532039153</t>
+        </is>
+      </c>
+      <c r="H234" t="n">
+        <v>0</v>
+      </c>
+      <c r="I234" t="n">
+        <v>0</v>
+      </c>
+      <c r="J234" t="inlineStr">
+        <is>
+          <t>multi_group</t>
+        </is>
+      </c>
+      <c r="L234" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="N234" t="inlineStr">
+        <is>
+          <t>Error code: 401 - [{'error': {'code': 401, 'message': 'Request had invalid authentication credentials. Expected OAuth 2 access token, login cookie or other valid authentication credential. See https://developers.google.com/identity/sign-in/web/devconsole-project.', 'status': 'UNAUTHENTICATED', 'details': [{'@type': 'type.googleapis.com/google.rpc.ErrorInfo', 'reason': 'ACCESS_TOKEN_TYPE_UNSUPPORTED', 'metadata': {'method': 'google.ai.generativelanguage.v1main.GenerativeService.GenerateContent', 'service': 'generativelanguage.googleapis.com'}}]}}]</t>
+        </is>
+      </c>
+    </row>
+    <row r="235">
+      <c r="A235" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B235" t="inlineStr">
+        <is>
+          <t>10:53:05</t>
+        </is>
+      </c>
+      <c r="C235" t="inlineStr">
+        <is>
+          <t>2100175696991846810</t>
+        </is>
+      </c>
+      <c r="D235" t="inlineStr">
+        <is>
+          <t>cryptowithgopal</t>
+        </is>
+      </c>
+      <c r="E235" t="inlineStr">
+        <is>
+          <t>#CRO
+crypto-com-chain:native is showing a double-bottom setup 👀📈
+Price is around $0.05543, with two reaction lows near $0.0547–$0.0548. The neckline sits around $0.0560, and price is approaching that resistance.
+🎯 Chart target: ~$0.0575
+🚀 A confirmed breakout above $0.0560 https://t.co/2tRIy3coAs</t>
+        </is>
+      </c>
+      <c r="F235" t="inlineStr">
+        <is>
+          <t>https://x.com/cryptowithgopal/status/2100175696991846810</t>
+        </is>
+      </c>
+      <c r="H235" t="n">
+        <v>0</v>
+      </c>
+      <c r="I235" t="n">
+        <v>0</v>
+      </c>
+      <c r="J235" t="inlineStr">
+        <is>
+          <t>multi_group</t>
+        </is>
+      </c>
+      <c r="L235" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="N235" t="inlineStr">
+        <is>
+          <t>Error code: 401 - [{'error': {'code': 401, 'message': 'Request had invalid authentication credentials. Expected OAuth 2 access token, login cookie or other valid authentication credential. See https://developers.google.com/identity/sign-in/web/devconsole-project.', 'status': 'UNAUTHENTICATED', 'details': [{'@type': 'type.googleapis.com/google.rpc.ErrorInfo', 'reason': 'ACCESS_TOKEN_TYPE_UNSUPPORTED', 'metadata': {'method': 'google.ai.generativelanguage.v1main.GenerativeService.GenerateContent', 'service': 'generativelanguage.googleapis.com'}}]}}]</t>
+        </is>
+      </c>
+    </row>
+    <row r="236">
+      <c r="A236" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B236" t="inlineStr">
+        <is>
+          <t>10:53:05</t>
+        </is>
+      </c>
+      <c r="C236" t="inlineStr">
+        <is>
+          <t>2100175683049669095</t>
+        </is>
+      </c>
+      <c r="D236" t="inlineStr">
+        <is>
+          <t>AdeboWalayyy</t>
+        </is>
+      </c>
+      <c r="E236" t="inlineStr">
+        <is>
+          <t>@omolaraeni81 @KaySoyemiEsq @CosyHomesOta More sales ma</t>
+        </is>
+      </c>
+      <c r="F236" t="inlineStr">
+        <is>
+          <t>https://x.com/AdeboWalayyy/status/2100175683049669095</t>
+        </is>
+      </c>
+      <c r="H236" t="n">
+        <v>0</v>
+      </c>
+      <c r="I236" t="n">
+        <v>0</v>
+      </c>
+      <c r="J236" t="inlineStr">
+        <is>
+          <t>multi_group</t>
+        </is>
+      </c>
+      <c r="L236" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="N236" t="inlineStr">
+        <is>
+          <t>Error code: 401 - [{'error': {'code': 401, 'message': 'Request had invalid authentication credentials. Expected OAuth 2 access token, login cookie or other valid authentication credential. See https://developers.google.com/identity/sign-in/web/devconsole-project.', 'status': 'UNAUTHENTICATED', 'details': [{'@type': 'type.googleapis.com/google.rpc.ErrorInfo', 'reason': 'ACCESS_TOKEN_TYPE_UNSUPPORTED', 'metadata': {'method': 'google.ai.generativelanguage.v1main.GenerativeService.GenerateContent', 'service': 'generativelanguage.googleapis.com'}}]}}]</t>
+        </is>
+      </c>
+    </row>
+    <row r="237">
+      <c r="A237" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B237" t="inlineStr">
+        <is>
+          <t>10:53:05</t>
+        </is>
+      </c>
+      <c r="C237" t="inlineStr">
+        <is>
+          <t>2100175680470192334</t>
+        </is>
+      </c>
+      <c r="D237" t="inlineStr">
+        <is>
+          <t>Tickeron</t>
+        </is>
+      </c>
+      <c r="E237" t="inlineStr">
+        <is>
+          <t>$CRDO https://t.co/BBc7q3fKFY</t>
+        </is>
+      </c>
+      <c r="F237" t="inlineStr">
+        <is>
+          <t>https://x.com/Tickeron/status/2100175680470192334</t>
+        </is>
+      </c>
+      <c r="H237" t="n">
+        <v>0</v>
+      </c>
+      <c r="I237" t="n">
+        <v>0</v>
+      </c>
+      <c r="J237" t="inlineStr">
+        <is>
+          <t>multi_group</t>
+        </is>
+      </c>
+      <c r="L237" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="N237" t="inlineStr">
+        <is>
+          <t>Error code: 401 - [{'error': {'code': 401, 'message': 'Request had invalid authentication credentials. Expected OAuth 2 access token, login cookie or other valid authentication credential. See https://developers.google.com/identity/sign-in/web/devconsole-project.', 'status': 'UNAUTHENTICATED', 'details': [{'@type': 'type.googleapis.com/google.rpc.ErrorInfo', 'reason': 'ACCESS_TOKEN_TYPE_UNSUPPORTED', 'metadata': {'method': 'google.ai.generativelanguage.v1main.GenerativeService.GenerateContent', 'service': 'generativelanguage.googleapis.com'}}]}}]</t>
+        </is>
+      </c>
+    </row>
+    <row r="238">
+      <c r="A238" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B238" t="inlineStr">
+        <is>
+          <t>10:53:05</t>
+        </is>
+      </c>
+      <c r="C238" t="inlineStr">
+        <is>
+          <t>2100175681342603357</t>
+        </is>
+      </c>
+      <c r="D238" t="inlineStr">
+        <is>
+          <t>andrii_rom</t>
+        </is>
+      </c>
+      <c r="E238" t="inlineStr">
+        <is>
+          <t>@T_Zahil I love your landing page and these design patterns!
+I've been doing it too for my sites, generating illustration like that, etc
+Can you share some design tips or prompts how you design like this? Is there some cool UI library that you use or is it all manual work?</t>
+        </is>
+      </c>
+      <c r="F238" t="inlineStr">
+        <is>
+          <t>https://x.com/andrii_rom/status/2100175681342603357</t>
+        </is>
+      </c>
+      <c r="H238" t="n">
+        <v>0</v>
+      </c>
+      <c r="I238" t="n">
+        <v>0</v>
+      </c>
+      <c r="J238" t="inlineStr">
+        <is>
+          <t>multi_group</t>
+        </is>
+      </c>
+      <c r="L238" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="N238" t="inlineStr">
+        <is>
+          <t>Error code: 401 - [{'error': {'code': 401, 'message': 'Request had invalid authentication credentials. Expected OAuth 2 access token, login cookie or other valid authentication credential. See https://developers.google.com/identity/sign-in/web/devconsole-project.', 'status': 'UNAUTHENTICATED', 'details': [{'@type': 'type.googleapis.com/google.rpc.ErrorInfo', 'reason': 'ACCESS_TOKEN_TYPE_UNSUPPORTED', 'metadata': {'method': 'google.ai.generativelanguage.v1main.GenerativeService.GenerateContent', 'service': 'generativelanguage.googleapis.com'}}]}}]</t>
+        </is>
+      </c>
+    </row>
+    <row r="239">
+      <c r="A239" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B239" t="inlineStr">
+        <is>
+          <t>10:53:05</t>
+        </is>
+      </c>
+      <c r="C239" t="inlineStr">
+        <is>
+          <t>2100175675151757704</t>
+        </is>
+      </c>
+      <c r="D239" t="inlineStr">
+        <is>
+          <t>TkakaBariga</t>
+        </is>
+      </c>
+      <c r="E239" t="inlineStr">
+        <is>
+          <t>@Deejayjasper006 @Midatlblog Blame those that will go to market and buy good goods for 5k and want to sell that same product for 40k</t>
+        </is>
+      </c>
+      <c r="F239" t="inlineStr">
+        <is>
+          <t>https://x.com/TkakaBariga/status/2100175675151757704</t>
+        </is>
+      </c>
+      <c r="H239" t="n">
+        <v>0</v>
+      </c>
+      <c r="I239" t="n">
+        <v>0</v>
+      </c>
+      <c r="J239" t="inlineStr">
+        <is>
+          <t>multi_group</t>
+        </is>
+      </c>
+      <c r="L239" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="N239" t="inlineStr">
+        <is>
+          <t>Error code: 401 - [{'error': {'code': 401, 'message': 'Request had invalid authentication credentials. Expected OAuth 2 access token, login cookie or other valid authentication credential. See https://developers.google.com/identity/sign-in/web/devconsole-project.', 'status': 'UNAUTHENTICATED', 'details': [{'@type': 'type.googleapis.com/google.rpc.ErrorInfo', 'reason': 'ACCESS_TOKEN_TYPE_UNSUPPORTED', 'metadata': {'method': 'google.ai.generativelanguage.v1main.GenerativeService.GenerateContent', 'service': 'generativelanguage.googleapis.com'}}]}}]</t>
+        </is>
+      </c>
+    </row>
+    <row r="240">
+      <c r="A240" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B240" t="inlineStr">
+        <is>
+          <t>10:53:05</t>
+        </is>
+      </c>
+      <c r="C240" t="inlineStr">
+        <is>
+          <t>2100175671733727512</t>
+        </is>
+      </c>
+      <c r="D240" t="inlineStr">
+        <is>
+          <t>strategist_ca</t>
+        </is>
+      </c>
+      <c r="E240" t="inlineStr">
+        <is>
+          <t>#COLPAL - Colgate Palmolive (India) Limited- A Global Leader in Consumer &amp;amp; Household Products- Is at Key #Technical Level &amp;amp; #Fundamental Level. FMCG sector has been Beaten Down Since Months Now &amp;amp; at Key Technical Level. If this Sector Bounce Backs &amp;amp; Became Dark Horse, this Stock https://t.co/xDvMaF1ym3</t>
+        </is>
+      </c>
+      <c r="F240" t="inlineStr">
+        <is>
+          <t>https://x.com/strategist_ca/status/2100175671733727512</t>
+        </is>
+      </c>
+      <c r="H240" t="n">
+        <v>0</v>
+      </c>
+      <c r="I240" t="n">
+        <v>0</v>
+      </c>
+      <c r="J240" t="inlineStr">
+        <is>
+          <t>multi_group</t>
+        </is>
+      </c>
+      <c r="L240" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="N240" t="inlineStr">
+        <is>
+          <t>Error code: 401 - [{'error': {'code': 401, 'message': 'Request had invalid authentication credentials. Expected OAuth 2 access token, login cookie or other valid authentication credential. See https://developers.google.com/identity/sign-in/web/devconsole-project.', 'status': 'UNAUTHENTICATED', 'details': [{'@type': 'type.googleapis.com/google.rpc.ErrorInfo', 'reason': 'ACCESS_TOKEN_TYPE_UNSUPPORTED', 'metadata': {'method': 'google.ai.generativelanguage.v1main.GenerativeService.GenerateContent', 'service': 'generativelanguage.googleapis.com'}}]}}]</t>
+        </is>
+      </c>
+    </row>
+    <row r="241">
+      <c r="A241" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B241" t="inlineStr">
+        <is>
+          <t>10:53:05</t>
+        </is>
+      </c>
+      <c r="C241" t="inlineStr">
+        <is>
+          <t>2100175658295218594</t>
+        </is>
+      </c>
+      <c r="D241" t="inlineStr">
+        <is>
+          <t>takumiautowork</t>
+        </is>
+      </c>
+      <c r="E241" t="inlineStr">
+        <is>
+          <t>会社員なら「1日3時間働いて月5万」より「自分が会社にいる間も集客が動く副業」を知ってほしい。
+これ、別に怪しい自動収益の話じゃない。
+Googleで「○○ 口コミ」「○○ 比較」と検索してる人に広告を出す。記事を読んでもらって、商品が売れたら成果報酬が入る。</t>
+        </is>
+      </c>
+      <c r="F241" t="inlineStr">
+        <is>
+          <t>https://x.com/takumiautowork/status/2100175658295218594</t>
+        </is>
+      </c>
+      <c r="H241" t="n">
+        <v>0</v>
+      </c>
+      <c r="I241" t="n">
+        <v>0</v>
+      </c>
+      <c r="J241" t="inlineStr">
+        <is>
+          <t>multi_group</t>
+        </is>
+      </c>
+      <c r="L241" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="N241" t="inlineStr">
+        <is>
+          <t>Error code: 401 - [{'error': {'code': 401, 'message': 'Request had invalid authentication credentials. Expected OAuth 2 access token, login cookie or other valid authentication credential. See https://developers.google.com/identity/sign-in/web/devconsole-project.', 'status': 'UNAUTHENTICATED', 'details': [{'@type': 'type.googleapis.com/google.rpc.ErrorInfo', 'reason': 'ACCESS_TOKEN_TYPE_UNSUPPORTED', 'metadata': {'method': 'google.ai.generativelanguage.v1main.GenerativeService.GenerateContent', 'service': 'generativelanguage.googleapis.com'}}]}}]</t>
+        </is>
+      </c>
+    </row>
+    <row r="242">
+      <c r="A242" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B242" t="inlineStr">
+        <is>
+          <t>10:53:06</t>
+        </is>
+      </c>
+      <c r="C242" t="inlineStr">
+        <is>
+          <t>2100175609318256957</t>
+        </is>
+      </c>
+      <c r="D242" t="inlineStr">
+        <is>
+          <t>takumiautowork</t>
+        </is>
+      </c>
+      <c r="E242" t="inlineStr">
+        <is>
+          <t>副業初心者が「動画編集、ライター、せどり」の3択で悩んでるなら、まだ知らない選択肢があります。
+僕なら会社員で平日1〜2時間しかないなら、「自分が作業した分だけ稼ぐ副業」だけでは選ばない。
+記事を1つ作る。そこにGoogle広告で「すでに商品を探してる人」を集める。売れたら成果報酬が入る。</t>
+        </is>
+      </c>
+      <c r="F242" t="inlineStr">
+        <is>
+          <t>https://x.com/takumiautowork/status/2100175609318256957</t>
+        </is>
+      </c>
+      <c r="H242" t="n">
+        <v>0</v>
+      </c>
+      <c r="I242" t="n">
+        <v>0</v>
+      </c>
+      <c r="J242" t="inlineStr">
+        <is>
+          <t>multi_group</t>
+        </is>
+      </c>
+      <c r="L242" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="N242" t="inlineStr">
+        <is>
+          <t>Error code: 401 - [{'error': {'code': 401, 'message': 'Request had invalid authentication credentials. Expected OAuth 2 access token, login cookie or other valid authentication credential. See https://developers.google.com/identity/sign-in/web/devconsole-project.', 'status': 'UNAUTHENTICATED', 'details': [{'@type': 'type.googleapis.com/google.rpc.ErrorInfo', 'reason': 'ACCESS_TOKEN_TYPE_UNSUPPORTED', 'metadata': {'service': 'generativelanguage.googleapis.com', 'method': 'google.ai.generativelanguage.v1main.GenerativeService.GenerateContent'}}]}}]</t>
+        </is>
+      </c>
+    </row>
+    <row r="243">
+      <c r="A243" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B243" t="inlineStr">
+        <is>
+          <t>10:53:06</t>
+        </is>
+      </c>
+      <c r="C243" t="inlineStr">
+        <is>
+          <t>2100175571854479547</t>
+        </is>
+      </c>
+      <c r="D243" t="inlineStr">
+        <is>
+          <t>Zoroaster711911</t>
+        </is>
+      </c>
+      <c r="E243" t="inlineStr">
+        <is>
+          <t>@GoatedExile @AltAfrikaner Unless the DNA splicing of Cro Magnon with homo erectus only happened 6000 years ago</t>
+        </is>
+      </c>
+      <c r="F243" t="inlineStr">
+        <is>
+          <t>https://x.com/Zoroaster711911/status/2100175571854479547</t>
+        </is>
+      </c>
+      <c r="H243" t="n">
+        <v>0</v>
+      </c>
+      <c r="I243" t="n">
+        <v>0</v>
+      </c>
+      <c r="J243" t="inlineStr">
+        <is>
+          <t>multi_group</t>
+        </is>
+      </c>
+      <c r="L243" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="N243" t="inlineStr">
+        <is>
+          <t>Error code: 401 - [{'error': {'code': 401, 'message': 'Request had invalid authentication credentials. Expected OAuth 2 access token, login cookie or other valid authentication credential. See https://developers.google.com/identity/sign-in/web/devconsole-project.', 'status': 'UNAUTHENTICATED', 'details': [{'@type': 'type.googleapis.com/google.rpc.ErrorInfo', 'reason': 'ACCESS_TOKEN_TYPE_UNSUPPORTED', 'metadata': {'method': 'google.ai.generativelanguage.v1main.GenerativeService.GenerateContent', 'service': 'generativelanguage.googleapis.com'}}]}}]</t>
+        </is>
+      </c>
+    </row>
+    <row r="244">
+      <c r="A244" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B244" t="inlineStr">
+        <is>
+          <t>10:53:06</t>
+        </is>
+      </c>
+      <c r="C244" t="inlineStr">
+        <is>
+          <t>2100175543689765121</t>
+        </is>
+      </c>
+      <c r="D244" t="inlineStr">
+        <is>
+          <t>__adwoasefah</t>
+        </is>
+      </c>
+      <c r="E244" t="inlineStr">
+        <is>
+          <t>@jesuisjemimaa i’ll keep clapping for others until it’s my turn🙏🏾</t>
+        </is>
+      </c>
+      <c r="F244" t="inlineStr">
+        <is>
+          <t>https://x.com/__adwoasefah/status/2100175543689765121</t>
+        </is>
+      </c>
+      <c r="H244" t="n">
+        <v>0</v>
+      </c>
+      <c r="I244" t="n">
+        <v>0</v>
+      </c>
+      <c r="J244" t="inlineStr">
+        <is>
+          <t>multi_group</t>
+        </is>
+      </c>
+      <c r="L244" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="N244" t="inlineStr">
+        <is>
+          <t>Error code: 401 - [{'error': {'code': 401, 'message': 'Request had invalid authentication credentials. Expected OAuth 2 access token, login cookie or other valid authentication credential. See https://developers.google.com/identity/sign-in/web/devconsole-project.', 'status': 'UNAUTHENTICATED', 'details': [{'@type': 'type.googleapis.com/google.rpc.ErrorInfo', 'reason': 'ACCESS_TOKEN_TYPE_UNSUPPORTED', 'metadata': {'method': 'google.ai.generativelanguage.v1main.GenerativeService.GenerateContent', 'service': 'generativelanguage.googleapis.com'}}]}}]</t>
+        </is>
+      </c>
+    </row>
+    <row r="245">
+      <c r="A245" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B245" t="inlineStr">
+        <is>
+          <t>10:53:06</t>
+        </is>
+      </c>
+      <c r="C245" t="inlineStr">
+        <is>
+          <t>2100175522160664800</t>
+        </is>
+      </c>
+      <c r="D245" t="inlineStr">
+        <is>
+          <t>A64076925</t>
+        </is>
+      </c>
+      <c r="E245" t="inlineStr">
+        <is>
+          <t>@warabimochi285 少しでますが、ジョージジェンセンの2026年のイヤーネックレスはどうでしょう！？産んだ年の記念になります🫶
+https://t.co/csMIErENqH</t>
+        </is>
+      </c>
+      <c r="F245" t="inlineStr">
+        <is>
+          <t>https://x.com/A64076925/status/2100175522160664800</t>
+        </is>
+      </c>
+      <c r="H245" t="n">
+        <v>0</v>
+      </c>
+      <c r="I245" t="n">
+        <v>0</v>
+      </c>
+      <c r="J245" t="inlineStr">
+        <is>
+          <t>multi_group</t>
+        </is>
+      </c>
+      <c r="L245" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="N245" t="inlineStr">
+        <is>
+          <t>Error code: 401 - [{'error': {'code': 401, 'message': 'Request had invalid authentication credentials. Expected OAuth 2 access token, login cookie or other valid authentication credential. See https://developers.google.com/identity/sign-in/web/devconsole-project.', 'status': 'UNAUTHENTICATED', 'details': [{'@type': 'type.googleapis.com/google.rpc.ErrorInfo', 'reason': 'ACCESS_TOKEN_TYPE_UNSUPPORTED', 'metadata': {'method': 'google.ai.generativelanguage.v1main.GenerativeService.GenerateContent', 'service': 'generativelanguage.googleapis.com'}}]}}]</t>
+        </is>
+      </c>
+    </row>
+    <row r="246">
+      <c r="A246" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B246" t="inlineStr">
+        <is>
+          <t>10:53:06</t>
+        </is>
+      </c>
+      <c r="C246" t="inlineStr">
+        <is>
+          <t>2100175502975664156</t>
+        </is>
+      </c>
+      <c r="D246" t="inlineStr">
+        <is>
+          <t>foto_bell</t>
+        </is>
+      </c>
+      <c r="E246" t="inlineStr">
+        <is>
+          <t>Moment two engineers in a cage inspect UK's most dangerous shipwreck off Kent, UK. Pics @Alamy_Editorial https://t.co/Q5f8MpSgdo @SunPictureDesk @Mailonlinepics @TelegraphPics @TimesPictures @guardianphotos @metropixdesk @Mirror_Pictures https://t.co/ATdDWByhLZ</t>
+        </is>
+      </c>
+      <c r="F246" t="inlineStr">
+        <is>
+          <t>https://x.com/foto_bell/status/2100175502975664156</t>
+        </is>
+      </c>
+      <c r="H246" t="n">
+        <v>0</v>
+      </c>
+      <c r="I246" t="n">
+        <v>0</v>
+      </c>
+      <c r="J246" t="inlineStr">
+        <is>
+          <t>multi_group</t>
+        </is>
+      </c>
+      <c r="L246" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="N246" t="inlineStr">
+        <is>
+          <t>Error code: 401 - [{'error': {'code': 401, 'message': 'Request had invalid authentication credentials. Expected OAuth 2 access token, login cookie or other valid authentication credential. See https://developers.google.com/identity/sign-in/web/devconsole-project.', 'status': 'UNAUTHENTICATED', 'details': [{'@type': 'type.googleapis.com/google.rpc.ErrorInfo', 'reason': 'ACCESS_TOKEN_TYPE_UNSUPPORTED', 'metadata': {'method': 'google.ai.generativelanguage.v1main.GenerativeService.GenerateContent', 'service': 'generativelanguage.googleapis.com'}}]}}]</t>
+        </is>
+      </c>
+    </row>
+    <row r="247">
+      <c r="A247" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B247" t="inlineStr">
+        <is>
+          <t>10:53:06</t>
+        </is>
+      </c>
+      <c r="C247" t="inlineStr">
+        <is>
+          <t>2100175480846463102</t>
+        </is>
+      </c>
+      <c r="D247" t="inlineStr">
+        <is>
+          <t>leedsboygrant23</t>
+        </is>
+      </c>
+      <c r="E247" t="inlineStr">
+        <is>
+          <t>@Johnyboylufc You’re my guy man. But this isn’t it. I’m from the south of England and I know people further than me that are supporters of this club. Yeah it’s a content creator, cool he’s gone Elland Road and yeah he went to the scum stadium. We move.</t>
+        </is>
+      </c>
+      <c r="F247" t="inlineStr">
+        <is>
+          <t>https://x.com/leedsboygrant23/status/2100175480846463102</t>
+        </is>
+      </c>
+      <c r="H247" t="n">
+        <v>0</v>
+      </c>
+      <c r="I247" t="n">
+        <v>0</v>
+      </c>
+      <c r="J247" t="inlineStr">
+        <is>
+          <t>multi_group</t>
+        </is>
+      </c>
+      <c r="L247" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="N247" t="inlineStr">
+        <is>
+          <t>Error code: 401 - [{'error': {'code': 401, 'message': 'Request had invalid authentication credentials. Expected OAuth 2 access token, login cookie or other valid authentication credential. See https://developers.google.com/identity/sign-in/web/devconsole-project.', 'status': 'UNAUTHENTICATED', 'details': [{'@type': 'type.googleapis.com/google.rpc.ErrorInfo', 'reason': 'ACCESS_TOKEN_TYPE_UNSUPPORTED', 'metadata': {'service': 'generativelanguage.googleapis.com', 'method': 'google.ai.generativelanguage.v1main.GenerativeService.GenerateContent'}}]}}]</t>
+        </is>
+      </c>
+    </row>
+    <row r="248">
+      <c r="A248" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B248" t="inlineStr">
+        <is>
+          <t>10:53:06</t>
+        </is>
+      </c>
+      <c r="C248" t="inlineStr">
+        <is>
+          <t>2100175406716403811</t>
+        </is>
+      </c>
+      <c r="D248" t="inlineStr">
+        <is>
+          <t>andrei_bsns</t>
+        </is>
+      </c>
+      <c r="E248" t="inlineStr">
+        <is>
+          <t>quanto costa partire per fare landing page e siti? molto poco: un abbonamento a claude o codex, poi netlify o vercel per il deploy.
+sotto i 100€ al mese stai molto chill e fai una buona quantità di pagine.
+#landingpage #vibecoding #tool #freelance https://t.co/HWDUbybqez</t>
+        </is>
+      </c>
+      <c r="F248" t="inlineStr">
+        <is>
+          <t>https://x.com/andrei_bsns/status/2100175406716403811</t>
+        </is>
+      </c>
+      <c r="H248" t="n">
+        <v>0</v>
+      </c>
+      <c r="I248" t="n">
+        <v>0</v>
+      </c>
+      <c r="J248" t="inlineStr">
+        <is>
+          <t>multi_group</t>
+        </is>
+      </c>
+      <c r="L248" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="N248" t="inlineStr">
+        <is>
+          <t>Error code: 401 - [{'error': {'code': 401, 'message': 'Request had invalid authentication credentials. Expected OAuth 2 access token, login cookie or other valid authentication credential. See https://developers.google.com/identity/sign-in/web/devconsole-project.', 'status': 'UNAUTHENTICATED', 'details': [{'@type': 'type.googleapis.com/google.rpc.ErrorInfo', 'reason': 'ACCESS_TOKEN_TYPE_UNSUPPORTED', 'metadata': {'method': 'google.ai.generativelanguage.v1main.GenerativeService.GenerateContent', 'service': 'generativelanguage.googleapis.com'}}]}}]</t>
+        </is>
+      </c>
+    </row>
+    <row r="249">
+      <c r="A249" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B249" t="inlineStr">
+        <is>
+          <t>10:53:06</t>
+        </is>
+      </c>
+      <c r="C249" t="inlineStr">
+        <is>
+          <t>2100175267570253869</t>
+        </is>
+      </c>
+      <c r="D249" t="inlineStr">
+        <is>
+          <t>weisskleee</t>
+        </is>
+      </c>
+      <c r="E249" t="inlineStr">
+        <is>
+          <t>Ich bin so stolz auf mich (n//n)🩷
+2026 konnte ich viele gesunde Routinen und Gewohnheiten entwickeln und vieles besser angehen.
+Ich freue mich sehr auf die Zukunft als Content Creator (und hoffentlich gutes Vorbild) und wie sich das auswirken wird 🍀</t>
+        </is>
+      </c>
+      <c r="F249" t="inlineStr">
+        <is>
+          <t>https://x.com/weisskleee/status/2100175267570253869</t>
+        </is>
+      </c>
+      <c r="H249" t="n">
+        <v>5</v>
+      </c>
+      <c r="I249" t="n">
+        <v>0</v>
+      </c>
+      <c r="J249" t="inlineStr">
+        <is>
+          <t>multi_group</t>
+        </is>
+      </c>
+      <c r="L249" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="N249" t="inlineStr">
+        <is>
+          <t>Error code: 401 - [{'error': {'code': 401, 'message': 'Request had invalid authentication credentials. Expected OAuth 2 access token, login cookie or other valid authentication credential. See https://developers.google.com/identity/sign-in/web/devconsole-project.', 'status': 'UNAUTHENTICATED', 'details': [{'@type': 'type.googleapis.com/google.rpc.ErrorInfo', 'reason': 'ACCESS_TOKEN_TYPE_UNSUPPORTED', 'metadata': {'method': 'google.ai.generativelanguage.v1main.GenerativeService.GenerateContent', 'service': 'generativelanguage.googleapis.com'}}]}}]</t>
+        </is>
+      </c>
+    </row>
+    <row r="250">
+      <c r="A250" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B250" t="inlineStr">
+        <is>
+          <t>10:53:07</t>
+        </is>
+      </c>
+      <c r="C250" t="inlineStr">
+        <is>
+          <t>2100175322826367418</t>
+        </is>
+      </c>
+      <c r="D250" t="inlineStr">
+        <is>
+          <t>sponton66</t>
+        </is>
+      </c>
+      <c r="E250" t="inlineStr">
+        <is>
+          <t>@poojeetstreet 💩😁</t>
+        </is>
+      </c>
+      <c r="F250" t="inlineStr">
+        <is>
+          <t>https://x.com/sponton66/status/2100175322826367418</t>
+        </is>
+      </c>
+      <c r="H250" t="n">
+        <v>0</v>
+      </c>
+      <c r="I250" t="n">
+        <v>0</v>
+      </c>
+      <c r="J250" t="inlineStr">
+        <is>
+          <t>multi_group</t>
+        </is>
+      </c>
+      <c r="L250" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="N250" t="inlineStr">
+        <is>
+          <t>Error code: 401 - [{'error': {'code': 401, 'message': 'Request had invalid authentication credentials. Expected OAuth 2 access token, login cookie or other valid authentication credential. See https://developers.google.com/identity/sign-in/web/devconsole-project.', 'status': 'UNAUTHENTICATED', 'details': [{'@type': 'type.googleapis.com/google.rpc.ErrorInfo', 'reason': 'ACCESS_TOKEN_TYPE_UNSUPPORTED', 'metadata': {'method': 'google.ai.generativelanguage.v1main.GenerativeService.GenerateContent', 'service': 'generativelanguage.googleapis.com'}}]}}]</t>
+        </is>
+      </c>
+    </row>
+    <row r="251">
+      <c r="A251" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B251" t="inlineStr">
+        <is>
+          <t>10:53:07</t>
+        </is>
+      </c>
+      <c r="C251" t="inlineStr">
+        <is>
+          <t>2100175297282715989</t>
+        </is>
+      </c>
+      <c r="D251" t="inlineStr">
+        <is>
+          <t>pixelcave_john</t>
+        </is>
+      </c>
+      <c r="E251" t="inlineStr">
+        <is>
+          <t>i have a problem every time i build a landing page.
+ai or by hand, same thing.
+design is fine but then i get to features.
+3 icons and some abstract blob just don't cut it.
+i want the product to actually move, like someone cared.
+yes, ai can generate a custom animation but it https://t.co/PAslOo2LmC</t>
+        </is>
+      </c>
+      <c r="F251" t="inlineStr">
+        <is>
+          <t>https://x.com/pixelcave_john/status/2100175297282715989</t>
+        </is>
+      </c>
+      <c r="H251" t="n">
+        <v>0</v>
+      </c>
+      <c r="I251" t="n">
+        <v>0</v>
+      </c>
+      <c r="J251" t="inlineStr">
+        <is>
+          <t>multi_group</t>
+        </is>
+      </c>
+      <c r="L251" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="N251" t="inlineStr">
+        <is>
+          <t>Error code: 401 - [{'error': {'code': 401, 'message': 'Request had invalid authentication credentials. Expected OAuth 2 access token, login cookie or other valid authentication credential. See https://developers.google.com/identity/sign-in/web/devconsole-project.', 'status': 'UNAUTHENTICATED', 'details': [{'@type': 'type.googleapis.com/google.rpc.ErrorInfo', 'reason': 'ACCESS_TOKEN_TYPE_UNSUPPORTED', 'metadata': {'method': 'google.ai.generativelanguage.v1main.GenerativeService.GenerateContent', 'service': 'generativelanguage.googleapis.com'}}]}}]</t>
+        </is>
+      </c>
+    </row>
+    <row r="252">
+      <c r="A252" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B252" t="inlineStr">
+        <is>
+          <t>10:53:07</t>
+        </is>
+      </c>
+      <c r="C252" t="inlineStr">
+        <is>
+          <t>2100175258716094778</t>
+        </is>
+      </c>
+      <c r="D252" t="inlineStr">
+        <is>
+          <t>CroAglo</t>
+        </is>
+      </c>
+      <c r="E252" t="inlineStr">
+        <is>
+          <t>@ZachBitango Is it possible for one to "scoot violently?"</t>
+        </is>
+      </c>
+      <c r="F252" t="inlineStr">
+        <is>
+          <t>https://x.com/CroAglo/status/2100175258716094778</t>
+        </is>
+      </c>
+      <c r="H252" t="n">
+        <v>0</v>
+      </c>
+      <c r="I252" t="n">
+        <v>0</v>
+      </c>
+      <c r="J252" t="inlineStr">
+        <is>
+          <t>multi_group</t>
+        </is>
+      </c>
+      <c r="L252" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="N252" t="inlineStr">
+        <is>
+          <t>Error code: 401 - [{'error': {'code': 401, 'message': 'Request had invalid authentication credentials. Expected OAuth 2 access token, login cookie or other valid authentication credential. See https://developers.google.com/identity/sign-in/web/devconsole-project.', 'status': 'UNAUTHENTICATED', 'details': [{'@type': 'type.googleapis.com/google.rpc.ErrorInfo', 'reason': 'ACCESS_TOKEN_TYPE_UNSUPPORTED', 'metadata': {'method': 'google.ai.generativelanguage.v1main.GenerativeService.GenerateContent', 'service': 'generativelanguage.googleapis.com'}}]}}]</t>
+        </is>
+      </c>
+    </row>
+    <row r="253">
+      <c r="A253" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B253" t="inlineStr">
+        <is>
+          <t>10:53:07</t>
+        </is>
+      </c>
+      <c r="C253" t="inlineStr">
+        <is>
+          <t>2100175220535333018</t>
+        </is>
+      </c>
+      <c r="D253" t="inlineStr">
+        <is>
+          <t>BigLambert3939</t>
+        </is>
+      </c>
+      <c r="E253" t="inlineStr">
+        <is>
+          <t>Two strategies can show similar APYs and still be completely different products.
+One might be supported by durable cash flows and diversified exposure.
+Another might depend on concentrated risk, thin liquidity, or assumptions that only work in a bull market.
+That’s why https://t.co/fkQLGOiZvi</t>
+        </is>
+      </c>
+      <c r="F253" t="inlineStr">
+        <is>
+          <t>https://x.com/BigLambert3939/status/2100175220535333018</t>
+        </is>
+      </c>
+      <c r="H253" t="n">
+        <v>0</v>
+      </c>
+      <c r="I253" t="n">
+        <v>0</v>
+      </c>
+      <c r="J253" t="inlineStr">
+        <is>
+          <t>multi_group</t>
+        </is>
+      </c>
+      <c r="L253" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="N253" t="inlineStr">
+        <is>
+          <t>Error code: 401 - [{'error': {'code': 401, 'message': 'Request had invalid authentication credentials. Expected OAuth 2 access token, login cookie or other valid authentication credential. See https://developers.google.com/identity/sign-in/web/devconsole-project.', 'status': 'UNAUTHENTICATED', 'details': [{'@type': 'type.googleapis.com/google.rpc.ErrorInfo', 'reason': 'ACCESS_TOKEN_TYPE_UNSUPPORTED', 'metadata': {'method': 'google.ai.generativelanguage.v1main.GenerativeService.GenerateContent', 'service': 'generativelanguage.googleapis.com'}}]}}]</t>
+        </is>
+      </c>
+    </row>
+    <row r="254">
+      <c r="A254" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B254" t="inlineStr">
+        <is>
+          <t>10:53:07</t>
+        </is>
+      </c>
+      <c r="C254" t="inlineStr">
+        <is>
+          <t>2100175150390112288</t>
+        </is>
+      </c>
+      <c r="D254" t="inlineStr">
+        <is>
+          <t>WorkZone7</t>
+        </is>
+      </c>
+      <c r="E254" t="inlineStr">
+        <is>
+          <t>@Ochekidoma @AfamDeluxo Never .psalm is a content creator and a guru in tech .. also a fanstribe podcast analyst</t>
+        </is>
+      </c>
+      <c r="F254" t="inlineStr">
+        <is>
+          <t>https://x.com/WorkZone7/status/2100175150390112288</t>
+        </is>
+      </c>
+      <c r="H254" t="n">
+        <v>3</v>
+      </c>
+      <c r="I254" t="n">
+        <v>0</v>
+      </c>
+      <c r="J254" t="inlineStr">
+        <is>
+          <t>multi_group</t>
+        </is>
+      </c>
+      <c r="L254" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="N254" t="inlineStr">
+        <is>
+          <t>Error code: 401 - [{'error': {'code': 401, 'message': 'Request had invalid authentication credentials. Expected OAuth 2 access token, login cookie or other valid authentication credential. See https://developers.google.com/identity/sign-in/web/devconsole-project.', 'status': 'UNAUTHENTICATED', 'details': [{'@type': 'type.googleapis.com/google.rpc.ErrorInfo', 'reason': 'ACCESS_TOKEN_TYPE_UNSUPPORTED', 'metadata': {'method': 'google.ai.generativelanguage.v1main.GenerativeService.GenerateContent', 'service': 'generativelanguage.googleapis.com'}}]}}]</t>
+        </is>
+      </c>
+    </row>
+    <row r="255">
+      <c r="A255" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B255" t="inlineStr">
+        <is>
+          <t>10:53:07</t>
+        </is>
+      </c>
+      <c r="C255" t="inlineStr">
+        <is>
+          <t>2100175180094222834</t>
+        </is>
+      </c>
+      <c r="D255" t="inlineStr">
+        <is>
+          <t>EngrShahid_</t>
+        </is>
+      </c>
+      <c r="E255" t="inlineStr">
+        <is>
+          <t>A small moment of carelessness can turn dangerous. Stay alert, even in everyday moments. 🙏⚠️
+Credit goes to the original content creator https://t.co/tCtLumb4uX</t>
+        </is>
+      </c>
+      <c r="F255" t="inlineStr">
+        <is>
+          <t>https://x.com/EngrShahid_/status/2100175180094222834</t>
+        </is>
+      </c>
+      <c r="H255" t="n">
+        <v>0</v>
+      </c>
+      <c r="I255" t="n">
+        <v>0</v>
+      </c>
+      <c r="J255" t="inlineStr">
+        <is>
+          <t>multi_group</t>
+        </is>
+      </c>
+      <c r="L255" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="N255" t="inlineStr">
+        <is>
+          <t>Error code: 401 - [{'error': {'code': 401, 'message': 'Request had invalid authentication credentials. Expected OAuth 2 access token, login cookie or other valid authentication credential. See https://developers.google.com/identity/sign-in/web/devconsole-project.', 'status': 'UNAUTHENTICATED', 'details': [{'@type': 'type.googleapis.com/google.rpc.ErrorInfo', 'reason': 'ACCESS_TOKEN_TYPE_UNSUPPORTED', 'metadata': {'method': 'google.ai.generativelanguage.v1main.GenerativeService.GenerateContent', 'service': 'generativelanguage.googleapis.com'}}]}}]</t>
+        </is>
+      </c>
+    </row>
+    <row r="256">
+      <c r="A256" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B256" t="inlineStr">
+        <is>
+          <t>10:53:07</t>
+        </is>
+      </c>
+      <c r="C256" t="inlineStr">
+        <is>
+          <t>2100175098145624537</t>
+        </is>
+      </c>
+      <c r="D256" t="inlineStr">
+        <is>
+          <t>pierreeliottlal</t>
+        </is>
+      </c>
+      <c r="E256" t="inlineStr">
+        <is>
+          <t>https://t.co/orMgvl0k17</t>
+        </is>
+      </c>
+      <c r="F256" t="inlineStr">
+        <is>
+          <t>https://x.com/pierreeliottlal/status/2100175098145624537</t>
+        </is>
+      </c>
+      <c r="H256" t="n">
+        <v>2</v>
+      </c>
+      <c r="I256" t="n">
+        <v>0</v>
+      </c>
+      <c r="J256" t="inlineStr">
+        <is>
+          <t>multi_group</t>
+        </is>
+      </c>
+      <c r="L256" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="N256" t="inlineStr">
+        <is>
+          <t>Error code: 401 - [{'error': {'code': 401, 'message': 'Request had invalid authentication credentials. Expected OAuth 2 access token, login cookie or other valid authentication credential. See https://developers.google.com/identity/sign-in/web/devconsole-project.', 'status': 'UNAUTHENTICATED', 'details': [{'@type': 'type.googleapis.com/google.rpc.ErrorInfo', 'reason': 'ACCESS_TOKEN_TYPE_UNSUPPORTED', 'metadata': {'method': 'google.ai.generativelanguage.v1main.GenerativeService.GenerateContent', 'service': 'generativelanguage.googleapis.com'}}]}}]</t>
+        </is>
+      </c>
+    </row>
+    <row r="257">
+      <c r="A257" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B257" t="inlineStr">
+        <is>
+          <t>10:53:07</t>
+        </is>
+      </c>
+      <c r="C257" t="inlineStr">
+        <is>
+          <t>2100175120555786450</t>
+        </is>
+      </c>
+      <c r="D257" t="inlineStr">
+        <is>
+          <t>EASL3616</t>
+        </is>
+      </c>
+      <c r="E257" t="inlineStr">
+        <is>
+          <t>Today is the day!!!!  Ratification Voting is taking place from 7 a.m. - 7 p.m.  Come by the office and Cast your Vote ✔️.
+Rain or Shine we will remain open 👍🏽
+Reminder this is ONLY for the CTA Bargaining Unit (Instructional only) https://t.co/t1V3wbOaDg</t>
+        </is>
+      </c>
+      <c r="F257" t="inlineStr">
+        <is>
+          <t>https://x.com/EASL3616/status/2100175120555786450</t>
+        </is>
+      </c>
+      <c r="H257" t="n">
+        <v>0</v>
+      </c>
+      <c r="I257" t="n">
+        <v>0</v>
+      </c>
+      <c r="J257" t="inlineStr">
+        <is>
+          <t>multi_group</t>
+        </is>
+      </c>
+      <c r="L257" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="N257" t="inlineStr">
+        <is>
+          <t>Error code: 401 - [{'error': {'code': 401, 'message': 'Request had invalid authentication credentials. Expected OAuth 2 access token, login cookie or other valid authentication credential. See https://developers.google.com/identity/sign-in/web/devconsole-project.', 'status': 'UNAUTHENTICATED', 'details': [{'@type': 'type.googleapis.com/google.rpc.ErrorInfo', 'reason': 'ACCESS_TOKEN_TYPE_UNSUPPORTED', 'metadata': {'method': 'google.ai.generativelanguage.v1main.GenerativeService.GenerateContent', 'service': 'generativelanguage.googleapis.com'}}]}}]</t>
+        </is>
+      </c>
+    </row>
+    <row r="258">
+      <c r="A258" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B258" t="inlineStr">
+        <is>
+          <t>10:53:07</t>
+        </is>
+      </c>
+      <c r="C258" t="inlineStr">
+        <is>
+          <t>2100175109910605980</t>
+        </is>
+      </c>
+      <c r="D258" t="inlineStr">
+        <is>
+          <t>Localmote</t>
+        </is>
+      </c>
+      <c r="E258" t="inlineStr">
+        <is>
+          <t>Canvify lets you turn any #Canva layout into a live #Shopify page in a few clicks. Design a section, product page, or full landing page in Canva, import it in our app...
+https://t.co/dBWXucYbn0
+#WebDesign #SaaS #LocalmoteBiz https://t.co/Pf6y4Z3rq7</t>
+        </is>
+      </c>
+      <c r="F258" t="inlineStr">
+        <is>
+          <t>https://x.com/Localmote/status/2100175109910605980</t>
+        </is>
+      </c>
+      <c r="H258" t="n">
+        <v>0</v>
+      </c>
+      <c r="I258" t="n">
+        <v>0</v>
+      </c>
+      <c r="J258" t="inlineStr">
+        <is>
+          <t>multi_group</t>
+        </is>
+      </c>
+      <c r="L258" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="N258" t="inlineStr">
+        <is>
+          <t>Error code: 401 - [{'error': {'code': 401, 'message': 'Request had invalid authentication credentials. Expected OAuth 2 access token, login cookie or other valid authentication credential. See https://developers.google.com/identity/sign-in/web/devconsole-project.', 'status': 'UNAUTHENTICATED', 'details': [{'@type': 'type.googleapis.com/google.rpc.ErrorInfo', 'reason': 'ACCESS_TOKEN_TYPE_UNSUPPORTED', 'metadata': {'method': 'google.ai.generativelanguage.v1main.GenerativeService.GenerateContent', 'service': 'generativelanguage.googleapis.com'}}]}}]</t>
+        </is>
+      </c>
+    </row>
+    <row r="259">
+      <c r="A259" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B259" t="inlineStr">
+        <is>
+          <t>10:53:07</t>
+        </is>
+      </c>
+      <c r="C259" t="inlineStr">
+        <is>
+          <t>2100175103405207826</t>
+        </is>
+      </c>
+      <c r="D259" t="inlineStr">
+        <is>
+          <t>CornelDaGreat</t>
+        </is>
+      </c>
+      <c r="E259" t="inlineStr">
+        <is>
+          <t>Need a newsletter that looks professional and converts?
+I design high-converting newsletters, landing pages and websites.
+Let’s build yours. 
+#fiverr 
+#GranHermanoGeneraciónDorada
+https://t.co/X6SG4j8VTk</t>
+        </is>
+      </c>
+      <c r="F259" t="inlineStr">
+        <is>
+          <t>https://x.com/CornelDaGreat/status/2100175103405207826</t>
+        </is>
+      </c>
+      <c r="H259" t="n">
+        <v>0</v>
+      </c>
+      <c r="I259" t="n">
+        <v>0</v>
+      </c>
+      <c r="J259" t="inlineStr">
+        <is>
+          <t>multi_group</t>
+        </is>
+      </c>
+      <c r="L259" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="N259" t="inlineStr">
+        <is>
+          <t>Error code: 401 - [{'error': {'code': 401, 'message': 'Request had invalid authentication credentials. Expected OAuth 2 access token, login cookie or other valid authentication credential. See https://developers.google.com/identity/sign-in/web/devconsole-project.', 'status': 'UNAUTHENTICATED', 'details': [{'@type': 'type.googleapis.com/google.rpc.ErrorInfo', 'reason': 'ACCESS_TOKEN_TYPE_UNSUPPORTED', 'metadata': {'method': 'google.ai.generativelanguage.v1main.GenerativeService.GenerateContent', 'service': 'generativelanguage.googleapis.com'}}]}}]</t>
+        </is>
+      </c>
+    </row>
+    <row r="260">
+      <c r="A260" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B260" t="inlineStr">
+        <is>
+          <t>10:53:08</t>
+        </is>
+      </c>
+      <c r="C260" t="inlineStr">
+        <is>
+          <t>2100175064616280207</t>
+        </is>
+      </c>
+      <c r="D260" t="inlineStr">
+        <is>
+          <t>ochuwa22</t>
+        </is>
+      </c>
+      <c r="E260" t="inlineStr">
+        <is>
+          <t>@Opemipo_wealthy What actually caused the traffic?</t>
+        </is>
+      </c>
+      <c r="F260" t="inlineStr">
+        <is>
+          <t>https://x.com/ochuwa22/status/2100175064616280207</t>
+        </is>
+      </c>
+      <c r="H260" t="n">
+        <v>0</v>
+      </c>
+      <c r="I260" t="n">
+        <v>0</v>
+      </c>
+      <c r="J260" t="inlineStr">
+        <is>
+          <t>multi_group</t>
+        </is>
+      </c>
+      <c r="L260" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="N260" t="inlineStr">
+        <is>
+          <t>Error code: 401 - [{'error': {'code': 401, 'message': 'Request had invalid authentication credentials. Expected OAuth 2 access token, login cookie or other valid authentication credential. See https://developers.google.com/identity/sign-in/web/devconsole-project.', 'status': 'UNAUTHENTICATED', 'details': [{'@type': 'type.googleapis.com/google.rpc.ErrorInfo', 'reason': 'ACCESS_TOKEN_TYPE_UNSUPPORTED', 'metadata': {'service': 'generativelanguage.googleapis.com', 'method': 'google.ai.generativelanguage.v1main.GenerativeService.GenerateContent'}}]}}]</t>
+        </is>
+      </c>
+    </row>
+    <row r="261">
+      <c r="A261" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B261" t="inlineStr">
+        <is>
+          <t>10:53:08</t>
+        </is>
+      </c>
+      <c r="C261" t="inlineStr">
+        <is>
+          <t>2100175021872140768</t>
+        </is>
+      </c>
+      <c r="D261" t="inlineStr">
+        <is>
+          <t>mightybeastlive</t>
+        </is>
+      </c>
+      <c r="E261" t="inlineStr">
+        <is>
+          <t>@WatchdogTh96012 The ad campaign was directed toward men to get more men watching female sports. You think men are going to be fired up about the stats of some women athletes? This was a shocking and risqué ad that started a conversation, thereby giving more attention to women's sports. Job done.</t>
+        </is>
+      </c>
+      <c r="F261" t="inlineStr">
+        <is>
+          <t>https://x.com/mightybeastlive/status/2100175021872140768</t>
+        </is>
+      </c>
+      <c r="H261" t="n">
+        <v>0</v>
+      </c>
+      <c r="I261" t="n">
+        <v>0</v>
+      </c>
+      <c r="J261" t="inlineStr">
+        <is>
+          <t>multi_group</t>
+        </is>
+      </c>
+      <c r="L261" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="N261" t="inlineStr">
+        <is>
+          <t>Error code: 401 - [{'error': {'code': 401, 'message': 'Request had invalid authentication credentials. Expected OAuth 2 access token, login cookie or other valid authentication credential. See https://developers.google.com/identity/sign-in/web/devconsole-project.', 'status': 'UNAUTHENTICATED', 'details': [{'@type': 'type.googleapis.com/google.rpc.ErrorInfo', 'reason': 'ACCESS_TOKEN_TYPE_UNSUPPORTED', 'metadata': {'method': 'google.ai.generativelanguage.v1main.GenerativeService.GenerateContent', 'service': 'generativelanguage.googleapis.com'}}]}}]</t>
+        </is>
+      </c>
+    </row>
+    <row r="262">
+      <c r="A262" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B262" t="inlineStr">
+        <is>
+          <t>10:53:08</t>
+        </is>
+      </c>
+      <c r="C262" t="inlineStr">
+        <is>
+          <t>2100174982462702071</t>
+        </is>
+      </c>
+      <c r="D262" t="inlineStr">
+        <is>
+          <t>RamSainyam</t>
+        </is>
+      </c>
+      <c r="E262" t="inlineStr">
+        <is>
+          <t>@winsttonxavier 2014 pachipoyina laddu nunchi 
+2019 BJP ni ammana bootulu titre CPI and CPM Kalisi 
+2024 lo fanboy behaviour gamanistunnam anni ghamanistunnam</t>
+        </is>
+      </c>
+      <c r="F262" t="inlineStr">
+        <is>
+          <t>https://x.com/RamSainyam/status/2100174982462702071</t>
+        </is>
+      </c>
+      <c r="H262" t="n">
+        <v>0</v>
+      </c>
+      <c r="I262" t="n">
+        <v>0</v>
+      </c>
+      <c r="J262" t="inlineStr">
+        <is>
+          <t>multi_group</t>
+        </is>
+      </c>
+      <c r="L262" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="N262" t="inlineStr">
+        <is>
+          <t>Error code: 401 - [{'error': {'code': 401, 'message': 'Request had invalid authentication credentials. Expected OAuth 2 access token, login cookie or other valid authentication credential. See https://developers.google.com/identity/sign-in/web/devconsole-project.', 'status': 'UNAUTHENTICATED', 'details': [{'@type': 'type.googleapis.com/google.rpc.ErrorInfo', 'reason': 'ACCESS_TOKEN_TYPE_UNSUPPORTED', 'metadata': {'method': 'google.ai.generativelanguage.v1main.GenerativeService.GenerateContent', 'service': 'generativelanguage.googleapis.com'}}]}}]</t>
+        </is>
+      </c>
+    </row>
+    <row r="263">
+      <c r="A263" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B263" t="inlineStr">
+        <is>
+          <t>10:53:08</t>
+        </is>
+      </c>
+      <c r="C263" t="inlineStr">
+        <is>
+          <t>2100174946118877217</t>
+        </is>
+      </c>
+      <c r="D263" t="inlineStr">
+        <is>
+          <t>Oboi_72by</t>
+        </is>
+      </c>
+      <c r="E263" t="inlineStr">
+        <is>
+          <t>@it_Rutie Na for clout you Dey whine content creator</t>
+        </is>
+      </c>
+      <c r="F263" t="inlineStr">
+        <is>
+          <t>https://x.com/Oboi_72by/status/2100174946118877217</t>
+        </is>
+      </c>
+      <c r="H263" t="n">
+        <v>0</v>
+      </c>
+      <c r="I263" t="n">
+        <v>0</v>
+      </c>
+      <c r="J263" t="inlineStr">
+        <is>
+          <t>multi_group</t>
+        </is>
+      </c>
+      <c r="L263" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="N263" t="inlineStr">
+        <is>
+          <t>Error code: 401 - [{'error': {'code': 401, 'message': 'Request had invalid authentication credentials. Expected OAuth 2 access token, login cookie or other valid authentication credential. See https://developers.google.com/identity/sign-in/web/devconsole-project.', 'status': 'UNAUTHENTICATED', 'details': [{'@type': 'type.googleapis.com/google.rpc.ErrorInfo', 'reason': 'ACCESS_TOKEN_TYPE_UNSUPPORTED', 'metadata': {'method': 'google.ai.generativelanguage.v1main.GenerativeService.GenerateContent', 'service': 'generativelanguage.googleapis.com'}}]}}]</t>
+        </is>
+      </c>
+    </row>
+    <row r="264">
+      <c r="A264" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B264" t="inlineStr">
+        <is>
+          <t>10:53:08</t>
+        </is>
+      </c>
+      <c r="C264" t="inlineStr">
+        <is>
+          <t>2100174936765563112</t>
+        </is>
+      </c>
+      <c r="D264" t="inlineStr">
+        <is>
+          <t>takumiautowork</t>
+        </is>
+      </c>
+      <c r="E264" t="inlineStr">
+        <is>
+          <t>副業初心者がPPCを知らないまま「何の副業やろう？」って悩んでるの、ちょっともったいないと思う。
+顔出しなしでもできる。大勢のフォロワーが前提じゃない。毎日SNS投稿する必要もない。自分の商品を最初から作る必要もない。</t>
+        </is>
+      </c>
+      <c r="F264" t="inlineStr">
+        <is>
+          <t>https://x.com/takumiautowork/status/2100174936765563112</t>
+        </is>
+      </c>
+      <c r="G264" t="inlineStr"/>
+      <c r="H264" t="n">
+        <v>0</v>
+      </c>
+      <c r="I264" t="n">
+        <v>0</v>
+      </c>
+      <c r="J264" t="inlineStr">
+        <is>
+          <t>multi_group</t>
+        </is>
+      </c>
+      <c r="K264" t="inlineStr"/>
+      <c r="L264" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="M264" t="inlineStr"/>
+      <c r="N264" t="inlineStr">
+        <is>
+          <t>Error code: 401 - [{'error': {'code': 401, 'message': 'Request had invalid authentication credentials. Expected OAuth 2 access token, login cookie or other valid authentication credential. See https://developers.google.com/identity/sign-in/web/devconsole-project.', 'status': 'UNAUTHENTICATED', 'details': [{'@type': 'type.googleapis.com/google.rpc.ErrorInfo', 'reason': 'ACCESS_TOKEN_TYPE_UNSUPPORTED', 'metadata': {'method': 'google.ai.generativelanguage.v1main.GenerativeService.GenerateContent', 'service': 'generativelanguage.googleapis.com'}}]}}]</t>
         </is>
       </c>
     </row>

</xml_diff>